<commit_message>
actualizacion 18 de mayo con cambios en GOB_EFF
</commit_message>
<xml_diff>
--- a/results/data/auditoria_normalizacion.xlsx
+++ b/results/data/auditoria_normalizacion.xlsx
@@ -3002,7 +3002,9 @@
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
+      <c r="L78" t="n">
+        <v>3.559770053525653</v>
+      </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
@@ -3036,7 +3038,9 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
+      <c r="L79" t="n">
+        <v>3.462256957637957</v>
+      </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
@@ -3070,7 +3074,9 @@
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
+      <c r="L80" t="n">
+        <v>3.362814898552893</v>
+      </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
@@ -3104,7 +3110,9 @@
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
+      <c r="L81" t="n">
+        <v>3.265301802665197</v>
+      </c>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
@@ -3138,7 +3146,9 @@
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
+      <c r="L82" t="n">
+        <v>3.164977138210421</v>
+      </c>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
@@ -3172,7 +3182,9 @@
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
+      <c r="L83" t="n">
+        <v>3.083118138507708</v>
+      </c>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
@@ -3206,7 +3218,9 @@
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
+      <c r="L84" t="n">
+        <v>3.01453376177852</v>
+      </c>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
@@ -3240,7 +3254,9 @@
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="L85" t="n">
+        <v>2.958474637102856</v>
+      </c>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
@@ -3276,7 +3292,9 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
+      <c r="L86" t="n">
+        <v>2.92100423308914</v>
+      </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
@@ -3312,7 +3330,9 @@
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
+      <c r="L87" t="n">
+        <v>2.874160130811208</v>
+      </c>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
@@ -3348,7 +3368,9 @@
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
+      <c r="L88" t="n">
+        <v>2.824056940931862</v>
+      </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
@@ -3384,7 +3406,9 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
+      <c r="L89" t="n">
+        <v>2.767141727220495</v>
+      </c>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
@@ -3420,7 +3444,9 @@
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
+      <c r="L90" t="n">
+        <v>2.704585640055734</v>
+      </c>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
@@ -3456,7 +3482,9 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
+      <c r="L91" t="n">
+        <v>2.628594192529179</v>
+      </c>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
@@ -3492,7 +3520,9 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
+      <c r="L92" t="n">
+        <v>2.540817894541739</v>
+      </c>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
@@ -3528,7 +3558,9 @@
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
+      <c r="L93" t="n">
+        <v>2.447514178478057</v>
+      </c>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
@@ -3564,7 +3596,9 @@
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+      <c r="L94" t="n">
+        <v>2.332851722434335</v>
+      </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
@@ -3600,7 +3634,9 @@
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
+      <c r="L95" t="n">
+        <v>2.271378185467958</v>
+      </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
@@ -3636,7 +3672,9 @@
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
+      <c r="L96" t="n">
+        <v>2.245841065182442</v>
+      </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
@@ -3672,7 +3710,9 @@
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
+      <c r="L97" t="n">
+        <v>2.258182190746167</v>
+      </c>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
@@ -3708,7 +3748,9 @@
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
+      <c r="L98" t="n">
+        <v>2.319502899964764</v>
+      </c>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
@@ -3744,7 +3786,9 @@
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
+      <c r="L99" t="n">
+        <v>2.378563124235711</v>
+      </c>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
@@ -3780,7 +3824,9 @@
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
+      <c r="L100" t="n">
+        <v>2.445749261340741</v>
+      </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
@@ -3816,7 +3862,9 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
+      <c r="L101" t="n">
+        <v>2.516761928155467</v>
+      </c>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
@@ -3852,7 +3900,9 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
+      <c r="L102" t="n">
+        <v>2.591863455544316</v>
+      </c>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
@@ -3888,7 +3938,9 @@
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
+      <c r="L103" t="n">
+        <v>2.675050858632044</v>
+      </c>
       <c r="M103" t="inlineStr"/>
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
@@ -3924,7 +3976,9 @@
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
+      <c r="L104" t="n">
+        <v>2.766756593535254</v>
+      </c>
       <c r="M104" t="inlineStr"/>
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
@@ -3960,7 +4014,9 @@
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
+      <c r="L105" t="n">
+        <v>2.865952799366765</v>
+      </c>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
@@ -4000,7 +4056,9 @@
         <v>0</v>
       </c>
       <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
+      <c r="L106" t="n">
+        <v>2.977081255619774</v>
+      </c>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="n">
         <v>0</v>
@@ -4046,7 +4104,9 @@
         <v>0</v>
       </c>
       <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
+      <c r="L107" t="n">
+        <v>3.080541913339261</v>
+      </c>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="n">
         <v>0</v>
@@ -4092,7 +4152,9 @@
         <v>0</v>
       </c>
       <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
+      <c r="L108" t="n">
+        <v>3.180493661295976</v>
+      </c>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="n">
         <v>0</v>
@@ -4138,7 +4200,9 @@
         <v>0</v>
       </c>
       <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
+      <c r="L109" t="n">
+        <v>3.276075825080323</v>
+      </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="n">
         <v>0</v>
@@ -4190,7 +4254,9 @@
         <v>36.05175557011729</v>
       </c>
       <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
+      <c r="L110" t="n">
+        <v>3.365278536457825</v>
+      </c>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="n">
         <v>0</v>
@@ -4244,7 +4310,9 @@
         <v>39.11655982955888</v>
       </c>
       <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
+      <c r="L111" t="n">
+        <v>3.457862318032019</v>
+      </c>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="n">
         <v>0</v>
@@ -4300,7 +4368,9 @@
         <v>37.40901422046526</v>
       </c>
       <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
+      <c r="L112" t="n">
+        <v>3.551977806391208</v>
+      </c>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="n">
         <v>0</v>
@@ -4354,7 +4424,9 @@
         <v>37.6768299111952</v>
       </c>
       <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
+      <c r="L113" t="n">
+        <v>3.648070945315732</v>
+      </c>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="n">
         <v>0</v>
@@ -4410,7 +4482,9 @@
         <v>40.95998746711458</v>
       </c>
       <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
+      <c r="L114" t="n">
+        <v>3.745292076286388</v>
+      </c>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="n">
         <v>0</v>
@@ -4464,7 +4538,9 @@
         <v>40.00101448795773</v>
       </c>
       <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
+      <c r="L115" t="n">
+        <v>3.842071255811641</v>
+      </c>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="n">
         <v>0</v>
@@ -4520,7 +4596,9 @@
         <v>42.53927997331215</v>
       </c>
       <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
+      <c r="L116" t="n">
+        <v>3.937812575856519</v>
+      </c>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="n">
         <v>0</v>
@@ -4574,7 +4652,9 @@
         <v>43.36718806455176</v>
       </c>
       <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
+      <c r="L117" t="n">
+        <v>4.039190298817401</v>
+      </c>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="n">
         <v>0</v>
@@ -4630,7 +4710,9 @@
         <v>42.90606636247666</v>
       </c>
       <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
+      <c r="L118" t="n">
+        <v>4.135729072026023</v>
+      </c>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="n">
         <v>6.617009865593446</v>
@@ -4684,7 +4766,9 @@
         <v>40.50251297395603</v>
       </c>
       <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
+      <c r="L119" t="n">
+        <v>4.290260834220383</v>
+      </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="n">
         <v>6.552703971541121</v>
@@ -4740,7 +4824,9 @@
         <v>43.09966546522338</v>
       </c>
       <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
+      <c r="L120" t="n">
+        <v>4.492201056386241</v>
+      </c>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="n">
         <v>6.47943270635322</v>
@@ -4794,7 +4880,9 @@
         <v>45.17406342670954</v>
       </c>
       <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
+      <c r="L121" t="n">
+        <v>4.730356743119993</v>
+      </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="n">
         <v>6.400187311146607</v>
@@ -4850,7 +4938,9 @@
         <v>42.97358243791349</v>
       </c>
       <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
+      <c r="L122" t="n">
+        <v>5.046873614333559</v>
+      </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="n">
         <v>6.234925664096019</v>
@@ -4904,7 +4994,9 @@
         <v>49.40316509340008</v>
       </c>
       <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
+      <c r="L123" t="n">
+        <v>5.252410701644767</v>
+      </c>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="n">
         <v>6.531064400585945</v>
@@ -4960,7 +5052,9 @@
         <v>46.68532061431296</v>
       </c>
       <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
+      <c r="L124" t="n">
+        <v>5.384951741667412</v>
+      </c>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="n">
         <v>6.382259561040986</v>
@@ -5014,7 +5108,9 @@
         <v>44.54748568370093</v>
       </c>
       <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
+      <c r="L125" t="n">
+        <v>5.43642549030184</v>
+      </c>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="n">
         <v>6.417270266653735</v>
@@ -5072,7 +5168,9 @@
         <v>46.21044300219359</v>
       </c>
       <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
+      <c r="L126" t="n">
+        <v>5.383489655901935</v>
+      </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="n">
         <v>6.336293698558523</v>
@@ -5130,7 +5228,9 @@
         <v>45.26051181084792</v>
       </c>
       <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="L127" t="n">
+        <v>5.334437875422402</v>
+      </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="n">
         <v>6.383028317900934</v>
@@ -5190,7 +5290,9 @@
         <v>46.45473170695444</v>
       </c>
       <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+      <c r="L128" t="n">
+        <v>5.266616764370014</v>
+      </c>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="n">
         <v>6.456372621653939</v>
@@ -5248,7 +5350,9 @@
         <v>47.72476062191947</v>
       </c>
       <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
+      <c r="L129" t="n">
+        <v>5.194225528988719</v>
+      </c>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="n">
         <v>6.543235690543376</v>
@@ -5308,7 +5412,9 @@
         <v>47.46777274013623</v>
       </c>
       <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
+      <c r="L130" t="n">
+        <v>5.106626997572721</v>
+      </c>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="n">
         <v>6.537509808588505</v>
@@ -5366,7 +5472,9 @@
         <v>45.70917871819964</v>
       </c>
       <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
+      <c r="L131" t="n">
+        <v>5.047925009821885</v>
+      </c>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="n">
         <v>6.488316933693232</v>
@@ -5426,7 +5534,9 @@
         <v>46.63209591586786</v>
       </c>
       <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
+      <c r="L132" t="n">
+        <v>5.006637298329766</v>
+      </c>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="n">
         <v>6.617159603644375</v>
@@ -5484,7 +5594,9 @@
         <v>49.6745928973661</v>
       </c>
       <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
+      <c r="L133" t="n">
+        <v>4.98321563089693</v>
+      </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>6.550681953204485</v>
@@ -5549,7 +5661,7 @@
         <v>22.84991617011906</v>
       </c>
       <c r="L134" t="n">
-        <v>0.9</v>
+        <v>4.982254005520306</v>
       </c>
       <c r="M134" t="n">
         <v>71.60141854805578</v>
@@ -5623,7 +5735,7 @@
         <v>22.43384803741664</v>
       </c>
       <c r="L135" t="n">
-        <v>0.8388888888888889</v>
+        <v>4.975863868256226</v>
       </c>
       <c r="M135" t="n">
         <v>70.40772918183548</v>
@@ -5699,7 +5811,7 @@
         <v>25.97498160412067</v>
       </c>
       <c r="L136" t="n">
-        <v>0.688888888888889</v>
+        <v>4.968821768640102</v>
       </c>
       <c r="M136" t="n">
         <v>72.29079143323273</v>
@@ -5773,7 +5885,7 @@
         <v>21.88944673443296</v>
       </c>
       <c r="L137" t="n">
-        <v>0.8107843137254902</v>
+        <v>4.965673977845193</v>
       </c>
       <c r="M137" t="n">
         <v>72.56921474351773</v>
@@ -5849,7 +5961,7 @@
         <v>21.77803915763171</v>
       </c>
       <c r="L138" t="n">
-        <v>0.7941176470588235</v>
+        <v>4.951574309350644</v>
       </c>
       <c r="M138" t="n">
         <v>73.24401070274702</v>
@@ -5927,7 +6039,7 @@
         <v>24.24223159953213</v>
       </c>
       <c r="L139" t="n">
-        <v>0.8937908496732024</v>
+        <v>5.001576668237532</v>
       </c>
       <c r="M139" t="n">
         <v>73.70939591035543</v>
@@ -6007,7 +6119,7 @@
         <v>22.35467255334805</v>
       </c>
       <c r="L140" t="n">
-        <v>1.04656862745098</v>
+        <v>5.100592514047802</v>
       </c>
       <c r="M140" t="n">
         <v>76.07237019829003</v>
@@ -6085,7 +6197,7 @@
         <v>20.43295559049504</v>
       </c>
       <c r="L141" t="n">
-        <v>0.9342691622103387</v>
+        <v>5.247216730183026</v>
       </c>
       <c r="M141" t="n">
         <v>76.03086600778188</v>
@@ -6165,7 +6277,7 @@
         <v>21.02317605818928</v>
       </c>
       <c r="L142" t="n">
-        <v>0.8413204442616207</v>
+        <v>5.462593300755228</v>
       </c>
       <c r="M142" t="n">
         <v>75.17399855773964</v>
@@ -6243,7 +6355,7 @@
         <v>24.59619209800186</v>
       </c>
       <c r="L143" t="n">
-        <v>0.8972027972027972</v>
+        <v>5.652452395776652</v>
       </c>
       <c r="M143" t="n">
         <v>76.43665393633636</v>
@@ -6323,7 +6435,7 @@
         <v>22.08768519433736</v>
       </c>
       <c r="L144" t="n">
-        <v>0.6972027972027972</v>
+        <v>5.836436605390112</v>
       </c>
       <c r="M144" t="n">
         <v>78.08806816880481</v>
@@ -6401,7 +6513,7 @@
         <v>23.49089420912626</v>
       </c>
       <c r="L145" t="n">
-        <v>0.6091346153846153</v>
+        <v>6.010345705406839</v>
       </c>
       <c r="M145" t="n">
         <v>78.66511371051087</v>
@@ -6481,7 +6593,7 @@
         <v>22.73912079667144</v>
       </c>
       <c r="L146" t="n">
-        <v>0.5858552631578947</v>
+        <v>6.168980248647733</v>
       </c>
       <c r="M146" t="n">
         <v>80.9309706354322</v>
@@ -6559,7 +6671,7 @@
         <v>22.33831089986639</v>
       </c>
       <c r="L147" t="n">
-        <v>0.7001409774436089</v>
+        <v>6.351046294260046</v>
       </c>
       <c r="M147" t="n">
         <v>82.52322794314793</v>
@@ -6639,7 +6751,7 @@
         <v>26.65739882607352</v>
       </c>
       <c r="L148" t="n">
-        <v>1.150140977443609</v>
+        <v>6.551430549491815</v>
       </c>
       <c r="M148" t="n">
         <v>84.76868087165163</v>
@@ -6717,7 +6829,7 @@
         <v>20.37890424987199</v>
       </c>
       <c r="L149" t="n">
-        <v>1.449248120300752</v>
+        <v>6.758738115121045</v>
       </c>
       <c r="M149" t="n">
         <v>85.39700590784228</v>
@@ -6797,7 +6909,7 @@
         <v>23.98255957526058</v>
       </c>
       <c r="L150" t="n">
-        <v>1.607142857142857</v>
+        <v>7.006076030660588</v>
       </c>
       <c r="M150" t="n">
         <v>87.66872650328276</v>
@@ -6875,7 +6987,7 @@
         <v>17.00660858624416</v>
       </c>
       <c r="L151" t="n">
-        <v>1.392857142857143</v>
+        <v>7.131958572200774</v>
       </c>
       <c r="M151" t="n">
         <v>89.24773532795588</v>
@@ -6955,7 +7067,7 @@
         <v>18.51507312705203</v>
       </c>
       <c r="L152" t="n">
-        <v>1.115079365079365</v>
+        <v>7.168123182068951</v>
       </c>
       <c r="M152" t="n">
         <v>90.36785562360491</v>
@@ -7033,7 +7145,7 @@
         <v>22.23544520524159</v>
       </c>
       <c r="L153" t="n">
-        <v>1.097222222222222</v>
+        <v>7.118313905782919</v>
       </c>
       <c r="M153" t="n">
         <v>90.15259557291911</v>
@@ -7113,7 +7225,7 @@
         <v>20.90352552439254</v>
       </c>
       <c r="L154" t="n">
-        <v>0.9543650793650793</v>
+        <v>6.937682480782353</v>
       </c>
       <c r="M154" t="n">
         <v>89.30372569807582</v>
@@ -7193,7 +7305,7 @@
         <v>19.20997891134999</v>
       </c>
       <c r="L155" t="n">
-        <v>0.7369737750172531</v>
+        <v>6.835693150350135</v>
       </c>
       <c r="M155" t="n">
         <v>88.79409990323373</v>
@@ -7273,7 +7385,7 @@
         <v>20.2796968623356</v>
       </c>
       <c r="L156" t="n">
-        <v>0.796001552795031</v>
+        <v>6.766559891195589</v>
       </c>
       <c r="M156" t="n">
         <v>89.20510718112509</v>
@@ -7353,7 +7465,7 @@
         <v>18.16721639333317</v>
       </c>
       <c r="L157" t="n">
-        <v>0.6154459972394755</v>
+        <v>6.750391327705373</v>
       </c>
       <c r="M157" t="n">
         <v>89.62374180480674</v>
@@ -7433,7 +7545,7 @@
         <v>18.89230770487385</v>
       </c>
       <c r="L158" t="n">
-        <v>0.8833031400966184</v>
+        <v>6.786067234566164</v>
       </c>
       <c r="M158" t="n">
         <v>89.95735929245305</v>
@@ -7513,7 +7625,7 @@
         <v>20.93220193263106</v>
       </c>
       <c r="L159" t="n">
-        <v>1.538194444444444</v>
+        <v>6.877964112551374</v>
       </c>
       <c r="M159" t="n">
         <v>91.53933219107782</v>
@@ -7593,7 +7705,7 @@
         <v>19.82028331640517</v>
       </c>
       <c r="L160" t="n">
-        <v>1.606944444444444</v>
+        <v>7.023651563673442</v>
       </c>
       <c r="M160" t="n">
         <v>92.69492342774645</v>
@@ -7673,7 +7785,7 @@
         <v>20.45488034645825</v>
       </c>
       <c r="L161" t="n">
-        <v>1.495833333333333</v>
+        <v>7.211512151729121</v>
       </c>
       <c r="M161" t="n">
         <v>91.99718819183596</v>
@@ -7753,7 +7865,7 @@
         <v>21.94832202701798</v>
       </c>
       <c r="L162" t="n">
-        <v>1.454166666666667</v>
+        <v>7.471922043709632</v>
       </c>
       <c r="M162" t="n">
         <v>91.01802175409797</v>
@@ -7833,7 +7945,7 @@
         <v>20.32592606318815</v>
       </c>
       <c r="L163" t="n">
-        <v>1.391666666666667</v>
+        <v>7.676361540957302</v>
       </c>
       <c r="M163" t="n">
         <v>91.137118674737</v>
@@ -7913,7 +8025,7 @@
         <v>18.58786689136544</v>
       </c>
       <c r="L164" t="n">
-        <v>1.080128205128205</v>
+        <v>7.853520002583915</v>
       </c>
       <c r="M164" t="n">
         <v>92.38543931526385</v>
@@ -7993,7 +8105,7 @@
         <v>23.36293094622431</v>
       </c>
       <c r="L165" t="n">
-        <v>1.071794871794872</v>
+        <v>7.990868800534436</v>
       </c>
       <c r="M165" t="n">
         <v>94.02384903400403</v>
@@ -8073,7 +8185,7 @@
         <v>23.50275922323679</v>
       </c>
       <c r="L166" t="n">
-        <v>1.071794871794872</v>
+        <v>8.090459308428599</v>
       </c>
       <c r="M166" t="n">
         <v>92.8584983200618</v>
@@ -8153,7 +8265,7 @@
         <v>22.96277506930686</v>
       </c>
       <c r="L167" t="n">
-        <v>0.5896520146520146</v>
+        <v>8.142834482392722</v>
       </c>
       <c r="M167" t="n">
         <v>92.56992824908228</v>
@@ -8233,7 +8345,7 @@
         <v>21.67958992718692</v>
       </c>
       <c r="L168" t="n">
-        <v>0.8011904761904761</v>
+        <v>8.150725723287294</v>
       </c>
       <c r="M168" t="n">
         <v>93.22826452664057</v>
@@ -8313,7 +8425,7 @@
         <v>24.60384111265572</v>
       </c>
       <c r="L169" t="n">
-        <v>1.126190476190476</v>
+        <v>8.119076275095445</v>
       </c>
       <c r="M169" t="n">
         <v>93.00248707528647</v>
@@ -8393,7 +8505,7 @@
         <v>23.53071333910281</v>
       </c>
       <c r="L170" t="n">
-        <v>1.876190476190476</v>
+        <v>8.032737049482087</v>
       </c>
       <c r="M170" t="n">
         <v>91.04535038119542</v>
@@ -8473,7 +8585,7 @@
         <v>24.40471183021596</v>
       </c>
       <c r="L171" t="n">
-        <v>1.889583333333333</v>
+        <v>7.955843348283997</v>
       </c>
       <c r="M171" t="n">
         <v>90.88697971861323</v>
@@ -8553,7 +8665,7 @@
         <v>25.80302780538268</v>
       </c>
       <c r="L172" t="n">
-        <v>2.577083333333333</v>
+        <v>7.873281226790117</v>
       </c>
       <c r="M172" t="n">
         <v>94.94428813348</v>
@@ -8633,7 +8745,7 @@
         <v>24.07725807123509</v>
       </c>
       <c r="L173" t="n">
-        <v>3.114583333333333</v>
+        <v>7.796387525592026</v>
       </c>
       <c r="M173" t="n">
         <v>96.16384819295274</v>
@@ -8713,7 +8825,7 @@
         <v>21.34583174640735</v>
       </c>
       <c r="L174" t="n">
-        <v>2.629329078799297</v>
+        <v>7.737738441246096</v>
       </c>
       <c r="M174" t="n">
         <v>96.6674779512479</v>
@@ -11352,7 +11464,9 @@
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
-      <c r="L78" t="inlineStr"/>
+      <c r="L78" t="n">
+        <v>75.15415197306064</v>
+      </c>
       <c r="M78" t="inlineStr"/>
       <c r="N78" t="inlineStr"/>
       <c r="O78" t="inlineStr"/>
@@ -11386,7 +11500,9 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
-      <c r="L79" t="inlineStr"/>
+      <c r="L79" t="n">
+        <v>75.8347564853275</v>
+      </c>
       <c r="M79" t="inlineStr"/>
       <c r="N79" t="inlineStr"/>
       <c r="O79" t="inlineStr"/>
@@ -11420,7 +11536,9 @@
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
-      <c r="L80" t="inlineStr"/>
+      <c r="L80" t="n">
+        <v>76.52882443083044</v>
+      </c>
       <c r="M80" t="inlineStr"/>
       <c r="N80" t="inlineStr"/>
       <c r="O80" t="inlineStr"/>
@@ -11454,7 +11572,9 @@
       <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
-      <c r="L81" t="inlineStr"/>
+      <c r="L81" t="n">
+        <v>77.20942894309732</v>
+      </c>
       <c r="M81" t="inlineStr"/>
       <c r="N81" t="inlineStr"/>
       <c r="O81" t="inlineStr"/>
@@ -11488,7 +11608,9 @@
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
-      <c r="L82" t="inlineStr"/>
+      <c r="L82" t="n">
+        <v>77.90965714012042</v>
+      </c>
       <c r="M82" t="inlineStr"/>
       <c r="N82" t="inlineStr"/>
       <c r="O82" t="inlineStr"/>
@@ -11522,7 +11644,9 @@
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr"/>
       <c r="K83" t="inlineStr"/>
-      <c r="L83" t="inlineStr"/>
+      <c r="L83" t="n">
+        <v>78.48100198421687</v>
+      </c>
       <c r="M83" t="inlineStr"/>
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
@@ -11556,7 +11680,9 @@
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
-      <c r="L84" t="inlineStr"/>
+      <c r="L84" t="n">
+        <v>78.95969498281325</v>
+      </c>
       <c r="M84" t="inlineStr"/>
       <c r="N84" t="inlineStr"/>
       <c r="O84" t="inlineStr"/>
@@ -11590,7 +11716,9 @@
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
-      <c r="L85" t="inlineStr"/>
+      <c r="L85" t="n">
+        <v>79.35096646138398</v>
+      </c>
       <c r="M85" t="inlineStr"/>
       <c r="N85" t="inlineStr"/>
       <c r="O85" t="inlineStr"/>
@@ -11626,7 +11754,9 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
-      <c r="L86" t="inlineStr"/>
+      <c r="L86" t="n">
+        <v>79.61249570333902</v>
+      </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
       <c r="O86" t="inlineStr"/>
@@ -11662,7 +11792,9 @@
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr"/>
-      <c r="L87" t="inlineStr"/>
+      <c r="L87" t="n">
+        <v>79.93944981235602</v>
+      </c>
       <c r="M87" t="inlineStr"/>
       <c r="N87" t="inlineStr"/>
       <c r="O87" t="inlineStr"/>
@@ -11698,7 +11830,9 @@
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
-      <c r="L88" t="inlineStr"/>
+      <c r="L88" t="n">
+        <v>80.28915111965652</v>
+      </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
       <c r="O88" t="inlineStr"/>
@@ -11734,7 +11868,9 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
-      <c r="L89" t="inlineStr"/>
+      <c r="L89" t="n">
+        <v>80.68639777576929</v>
+      </c>
       <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr"/>
       <c r="O89" t="inlineStr"/>
@@ -11770,7 +11906,9 @@
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
-      <c r="L90" t="inlineStr"/>
+      <c r="L90" t="n">
+        <v>81.12301559419166</v>
+      </c>
       <c r="M90" t="inlineStr"/>
       <c r="N90" t="inlineStr"/>
       <c r="O90" t="inlineStr"/>
@@ -11806,7 +11944,9 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
-      <c r="L91" t="inlineStr"/>
+      <c r="L91" t="n">
+        <v>81.65340714426436</v>
+      </c>
       <c r="M91" t="inlineStr"/>
       <c r="N91" t="inlineStr"/>
       <c r="O91" t="inlineStr"/>
@@ -11842,7 +11982,9 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
-      <c r="L92" t="inlineStr"/>
+      <c r="L92" t="n">
+        <v>82.26605249139945</v>
+      </c>
       <c r="M92" t="inlineStr"/>
       <c r="N92" t="inlineStr"/>
       <c r="O92" t="inlineStr"/>
@@ -11878,7 +12020,9 @@
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
-      <c r="L93" t="inlineStr"/>
+      <c r="L93" t="n">
+        <v>82.91727712524089</v>
+      </c>
       <c r="M93" t="inlineStr"/>
       <c r="N93" t="inlineStr"/>
       <c r="O93" t="inlineStr"/>
@@ -11914,7 +12058,9 @@
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
+      <c r="L94" t="n">
+        <v>83.7175776824177</v>
+      </c>
       <c r="M94" t="inlineStr"/>
       <c r="N94" t="inlineStr"/>
       <c r="O94" t="inlineStr"/>
@@ -11950,7 +12096,9 @@
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
-      <c r="L95" t="inlineStr"/>
+      <c r="L95" t="n">
+        <v>84.14663971007094</v>
+      </c>
       <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr"/>
       <c r="O95" t="inlineStr"/>
@@ -11986,7 +12134,9 @@
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
-      <c r="L96" t="inlineStr"/>
+      <c r="L96" t="n">
+        <v>84.324879146922</v>
+      </c>
       <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr"/>
       <c r="O96" t="inlineStr"/>
@@ -12022,7 +12172,9 @@
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
-      <c r="L97" t="inlineStr"/>
+      <c r="L97" t="n">
+        <v>84.23874276012532</v>
+      </c>
       <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr"/>
       <c r="O97" t="inlineStr"/>
@@ -12058,7 +12210,9 @@
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
-      <c r="L98" t="inlineStr"/>
+      <c r="L98" t="n">
+        <v>83.81074741232457</v>
+      </c>
       <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr"/>
       <c r="O98" t="inlineStr"/>
@@ -12094,7 +12248,9 @@
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
-      <c r="L99" t="inlineStr"/>
+      <c r="L99" t="n">
+        <v>83.39852939413556</v>
+      </c>
       <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr"/>
       <c r="O99" t="inlineStr"/>
@@ -12130,7 +12286,9 @@
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
-      <c r="L100" t="inlineStr"/>
+      <c r="L100" t="n">
+        <v>82.92959557904956</v>
+      </c>
       <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr"/>
       <c r="O100" t="inlineStr"/>
@@ -12166,7 +12324,9 @@
       <c r="I101" t="inlineStr"/>
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
+      <c r="L101" t="n">
+        <v>82.43395403447313</v>
+      </c>
       <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr"/>
       <c r="O101" t="inlineStr"/>
@@ -12202,7 +12362,9 @@
       <c r="I102" t="inlineStr"/>
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
-      <c r="L102" t="inlineStr"/>
+      <c r="L102" t="n">
+        <v>81.9097737902334</v>
+      </c>
       <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr"/>
       <c r="O102" t="inlineStr"/>
@@ -12238,7 +12400,9 @@
       <c r="I103" t="inlineStr"/>
       <c r="J103" t="inlineStr"/>
       <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
+      <c r="L103" t="n">
+        <v>81.32915719315113</v>
+      </c>
       <c r="M103" t="inlineStr"/>
       <c r="N103" t="inlineStr"/>
       <c r="O103" t="inlineStr"/>
@@ -12274,7 +12438,9 @@
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
+      <c r="L104" t="n">
+        <v>80.68908586316529</v>
+      </c>
       <c r="M104" t="inlineStr"/>
       <c r="N104" t="inlineStr"/>
       <c r="O104" t="inlineStr"/>
@@ -12310,7 +12476,9 @@
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
-      <c r="L105" t="inlineStr"/>
+      <c r="L105" t="n">
+        <v>79.99673388034614</v>
+      </c>
       <c r="M105" t="inlineStr"/>
       <c r="N105" t="inlineStr"/>
       <c r="O105" t="inlineStr"/>
@@ -12350,7 +12518,9 @@
         <v>0</v>
       </c>
       <c r="K106" t="inlineStr"/>
-      <c r="L106" t="inlineStr"/>
+      <c r="L106" t="n">
+        <v>79.22109930451279</v>
+      </c>
       <c r="M106" t="inlineStr"/>
       <c r="N106" t="n">
         <v>0</v>
@@ -12396,7 +12566,9 @@
         <v>0</v>
       </c>
       <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
+      <c r="L107" t="n">
+        <v>78.49898306109992</v>
+      </c>
       <c r="M107" t="inlineStr"/>
       <c r="N107" t="n">
         <v>0</v>
@@ -12442,7 +12614,9 @@
         <v>0</v>
       </c>
       <c r="K108" t="inlineStr"/>
-      <c r="L108" t="inlineStr"/>
+      <c r="L108" t="n">
+        <v>77.80135768012906</v>
+      </c>
       <c r="M108" t="inlineStr"/>
       <c r="N108" t="n">
         <v>0</v>
@@ -12488,7 +12662,9 @@
         <v>0</v>
       </c>
       <c r="K109" t="inlineStr"/>
-      <c r="L109" t="inlineStr"/>
+      <c r="L109" t="n">
+        <v>77.13423034331699</v>
+      </c>
       <c r="M109" t="inlineStr"/>
       <c r="N109" t="n">
         <v>0</v>
@@ -12540,7 +12716,9 @@
         <v>30.29059231412641</v>
       </c>
       <c r="K110" t="inlineStr"/>
-      <c r="L110" t="inlineStr"/>
+      <c r="L110" t="n">
+        <v>76.51162917044594</v>
+      </c>
       <c r="M110" t="inlineStr"/>
       <c r="N110" t="n">
         <v>0</v>
@@ -12594,7 +12772,9 @@
         <v>32.86563297101727</v>
       </c>
       <c r="K111" t="inlineStr"/>
-      <c r="L111" t="inlineStr"/>
+      <c r="L111" t="n">
+        <v>75.86542940693214</v>
+      </c>
       <c r="M111" t="inlineStr"/>
       <c r="N111" t="n">
         <v>0</v>
@@ -12650,7 +12830,9 @@
         <v>31.43095754162698</v>
       </c>
       <c r="K112" t="inlineStr"/>
-      <c r="L112" t="inlineStr"/>
+      <c r="L112" t="n">
+        <v>75.20853890962667</v>
+      </c>
       <c r="M112" t="inlineStr"/>
       <c r="N112" t="n">
         <v>0</v>
@@ -12704,7 +12886,9 @@
         <v>31.65597559622488</v>
       </c>
       <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
+      <c r="L113" t="n">
+        <v>74.53784515967907</v>
+      </c>
       <c r="M113" t="inlineStr"/>
       <c r="N113" t="n">
         <v>0</v>
@@ -12760,7 +12944,9 @@
         <v>34.4144761312676</v>
       </c>
       <c r="K114" t="inlineStr"/>
-      <c r="L114" t="inlineStr"/>
+      <c r="L114" t="n">
+        <v>73.85927845205937</v>
+      </c>
       <c r="M114" t="inlineStr"/>
       <c r="N114" t="n">
         <v>0</v>
@@ -12814,7 +13000,9 @@
         <v>33.60874950041301</v>
       </c>
       <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
+      <c r="L115" t="n">
+        <v>73.18379639830289</v>
+      </c>
       <c r="M115" t="inlineStr"/>
       <c r="N115" t="n">
         <v>0</v>
@@ -12870,7 +13058,9 @@
         <v>35.74139363343876</v>
       </c>
       <c r="K116" t="inlineStr"/>
-      <c r="L116" t="inlineStr"/>
+      <c r="L116" t="n">
+        <v>72.5155582110139</v>
+      </c>
       <c r="M116" t="inlineStr"/>
       <c r="N116" t="n">
         <v>0</v>
@@ -12924,7 +13114,9 @@
         <v>36.43699988253062</v>
       </c>
       <c r="K117" t="inlineStr"/>
-      <c r="L117" t="inlineStr"/>
+      <c r="L117" t="n">
+        <v>71.80798006407474</v>
+      </c>
       <c r="M117" t="inlineStr"/>
       <c r="N117" t="n">
         <v>0</v>
@@ -12980,7 +13172,9 @@
         <v>36.04956661433409</v>
       </c>
       <c r="K118" t="inlineStr"/>
-      <c r="L118" t="inlineStr"/>
+      <c r="L118" t="n">
+        <v>71.13417595544334</v>
+      </c>
       <c r="M118" t="inlineStr"/>
       <c r="N118" t="n">
         <v>26.7128482831499</v>
@@ -13034,7 +13228,9 @@
         <v>34.03010723862307</v>
       </c>
       <c r="K119" t="inlineStr"/>
-      <c r="L119" t="inlineStr"/>
+      <c r="L119" t="n">
+        <v>70.05560272709295</v>
+      </c>
       <c r="M119" t="inlineStr"/>
       <c r="N119" t="n">
         <v>26.45324558851526</v>
@@ -13090,7 +13286,9 @@
         <v>36.21222808257455</v>
       </c>
       <c r="K120" t="inlineStr"/>
-      <c r="L120" t="inlineStr"/>
+      <c r="L120" t="n">
+        <v>68.64613638656625</v>
+      </c>
       <c r="M120" t="inlineStr"/>
       <c r="N120" t="n">
         <v>26.15744971844165</v>
@@ -13144,7 +13342,9 @@
         <v>37.9551319149947</v>
       </c>
       <c r="K121" t="inlineStr"/>
-      <c r="L121" t="inlineStr"/>
+      <c r="L121" t="n">
+        <v>66.98389980657208</v>
+      </c>
       <c r="M121" t="inlineStr"/>
       <c r="N121" t="n">
         <v>25.83753630403077</v>
@@ -13200,7 +13400,9 @@
         <v>36.10629344728205</v>
       </c>
       <c r="K122" t="inlineStr"/>
-      <c r="L122" t="inlineStr"/>
+      <c r="L122" t="n">
+        <v>64.77473180923307</v>
+      </c>
       <c r="M122" t="inlineStr"/>
       <c r="N122" t="n">
         <v>25.17037554798588</v>
@@ -13254,7 +13456,9 @@
         <v>41.50841225918126</v>
       </c>
       <c r="K123" t="inlineStr"/>
-      <c r="L123" t="inlineStr"/>
+      <c r="L123" t="n">
+        <v>63.34016071097457</v>
+      </c>
       <c r="M123" t="inlineStr"/>
       <c r="N123" t="n">
         <v>26.36588670775496</v>
@@ -13310,7 +13514,9 @@
         <v>39.22488631745249</v>
       </c>
       <c r="K124" t="inlineStr"/>
-      <c r="L124" t="inlineStr"/>
+      <c r="L124" t="n">
+        <v>62.41507440252788</v>
+      </c>
       <c r="M124" t="inlineStr"/>
       <c r="N124" t="n">
         <v>25.7651620325158</v>
@@ -13364,7 +13570,9 @@
         <v>37.42868290671642</v>
       </c>
       <c r="K125" t="inlineStr"/>
-      <c r="L125" t="inlineStr"/>
+      <c r="L125" t="n">
+        <v>62.05580711370926</v>
+      </c>
       <c r="M125" t="inlineStr"/>
       <c r="N125" t="n">
         <v>25.9065001423745</v>
@@ -13422,7 +13630,9 @@
         <v>38.82589536901344</v>
       </c>
       <c r="K126" t="inlineStr"/>
-      <c r="L126" t="inlineStr"/>
+      <c r="L126" t="n">
+        <v>62.42527920794654</v>
+      </c>
       <c r="M126" t="inlineStr"/>
       <c r="N126" t="n">
         <v>25.57959798838723</v>
@@ -13480,7 +13690,9 @@
         <v>38.02776562502466</v>
       </c>
       <c r="K127" t="inlineStr"/>
-      <c r="L127" t="inlineStr"/>
+      <c r="L127" t="n">
+        <v>62.7676420754689</v>
+      </c>
       <c r="M127" t="inlineStr"/>
       <c r="N127" t="n">
         <v>25.7682655015726</v>
@@ -13540,7 +13752,9 @@
         <v>39.0311461105055</v>
       </c>
       <c r="K128" t="inlineStr"/>
-      <c r="L128" t="inlineStr"/>
+      <c r="L128" t="n">
+        <v>63.24100776844585</v>
+      </c>
       <c r="M128" t="inlineStr"/>
       <c r="N128" t="n">
         <v>26.06435622810677</v>
@@ -13598,7 +13812,9 @@
         <v>40.09822113866988</v>
       </c>
       <c r="K129" t="inlineStr"/>
-      <c r="L129" t="inlineStr"/>
+      <c r="L129" t="n">
+        <v>63.74627119999383</v>
+      </c>
       <c r="M129" t="inlineStr"/>
       <c r="N129" t="n">
         <v>26.41502216752414</v>
@@ -13658,7 +13874,9 @@
         <v>39.88230058130264</v>
       </c>
       <c r="K130" t="inlineStr"/>
-      <c r="L130" t="inlineStr"/>
+      <c r="L130" t="n">
+        <v>64.35767580372359</v>
+      </c>
       <c r="M130" t="inlineStr"/>
       <c r="N130" t="n">
         <v>26.39190679984983</v>
@@ -13716,7 +13934,9 @@
         <v>38.40473440672515</v>
       </c>
       <c r="K131" t="inlineStr"/>
-      <c r="L131" t="inlineStr"/>
+      <c r="L131" t="n">
+        <v>64.76739346655185</v>
+      </c>
       <c r="M131" t="inlineStr"/>
       <c r="N131" t="n">
         <v>26.19331531662986</v>
@@ -13776,7 +13996,9 @@
         <v>39.18016706269922</v>
       </c>
       <c r="K132" t="inlineStr"/>
-      <c r="L132" t="inlineStr"/>
+      <c r="L132" t="n">
+        <v>65.05556607031239</v>
+      </c>
       <c r="M132" t="inlineStr"/>
       <c r="N132" t="n">
         <v>26.7134527751966</v>
@@ -13834,7 +14056,9 @@
         <v>41.73646520203068</v>
       </c>
       <c r="K133" t="inlineStr"/>
-      <c r="L133" t="inlineStr"/>
+      <c r="L133" t="n">
+        <v>65.21904044669731</v>
+      </c>
       <c r="M133" t="inlineStr"/>
       <c r="N133" t="n">
         <v>26.44508270676815</v>
@@ -13899,7 +14123,7 @@
         <v>82.70112145333562</v>
       </c>
       <c r="L134" t="n">
-        <v>30.22711122236004</v>
+        <v>65.2257522279661</v>
       </c>
       <c r="M134" t="n">
         <v>71.60141854805578</v>
@@ -13973,7 +14197,7 @@
         <v>81.1952384155465</v>
       </c>
       <c r="L135" t="n">
-        <v>28.17465305294053</v>
+        <v>65.27035296816766</v>
       </c>
       <c r="M135" t="n">
         <v>70.40772918183548</v>
@@ -14049,7 +14273,7 @@
         <v>94.01172820054809</v>
       </c>
       <c r="L136" t="n">
-        <v>23.1368011825472</v>
+        <v>65.31950415889682</v>
       </c>
       <c r="M136" t="n">
         <v>72.29079143323273</v>
@@ -14123,7 +14347,7 @@
         <v>79.22487677648353</v>
       </c>
       <c r="L137" t="n">
-        <v>27.23074180925028</v>
+        <v>65.34147454758342</v>
       </c>
       <c r="M137" t="n">
         <v>72.56921474351773</v>
@@ -14199,7 +14423,7 @@
         <v>78.82165728669344</v>
       </c>
       <c r="L138" t="n">
-        <v>26.67098049031768</v>
+        <v>65.43988489863935</v>
       </c>
       <c r="M138" t="n">
         <v>73.24401070274702</v>
@@ -14277,7 +14501,7 @@
         <v>87.74035427029538</v>
       </c>
       <c r="L139" t="n">
-        <v>30.01857269177731</v>
+        <v>65.09088735351374</v>
       </c>
       <c r="M139" t="n">
         <v>73.70939591035543</v>
@@ -14357,7 +14581,7 @@
         <v>80.9086771312366</v>
       </c>
       <c r="L140" t="n">
-        <v>35.14971811532608</v>
+        <v>64.39979421539816</v>
       </c>
       <c r="M140" t="n">
         <v>76.07237019829003</v>
@@ -14435,7 +14659,7 @@
         <v>73.95337161673879</v>
       </c>
       <c r="L141" t="n">
-        <v>31.37806430861449</v>
+        <v>63.37641266648133</v>
       </c>
       <c r="M141" t="n">
         <v>76.03086600778188</v>
@@ -14515,7 +14739,7 @@
         <v>76.089567400549</v>
       </c>
       <c r="L142" t="n">
-        <v>28.25631849149041</v>
+        <v>61.87316569812717</v>
       </c>
       <c r="M142" t="n">
         <v>75.17399855773964</v>
@@ -14593,7 +14817,7 @@
         <v>89.02145000630114</v>
       </c>
       <c r="L143" t="n">
-        <v>30.13316526673499</v>
+        <v>60.54802105380879</v>
       </c>
       <c r="M143" t="n">
         <v>76.43665393633636</v>
@@ -14673,7 +14897,7 @@
         <v>79.94236487697448</v>
       </c>
       <c r="L144" t="n">
-        <v>23.41602943954387</v>
+        <v>59.26388088669739</v>
       </c>
       <c r="M144" t="n">
         <v>78.08806816880481</v>
@@ -14751,7 +14975,7 @@
         <v>85.0210250476506</v>
       </c>
       <c r="L145" t="n">
-        <v>20.45819974291141</v>
+        <v>58.05006117234873</v>
       </c>
       <c r="M145" t="n">
         <v>78.66511371051087</v>
@@ -14831,7 +15055,7 @@
         <v>82.30011772239232</v>
       </c>
       <c r="L146" t="n">
-        <v>19.67634688853188</v>
+        <v>56.94285208470484</v>
       </c>
       <c r="M146" t="n">
         <v>80.9309706354322</v>
@@ -14909,7 +15133,7 @@
         <v>80.84945909815104</v>
       </c>
       <c r="L147" t="n">
-        <v>23.51471021835538</v>
+        <v>55.67209997652607</v>
       </c>
       <c r="M147" t="n">
         <v>82.52322794314793</v>
@@ -14989,7 +15213,7 @@
         <v>96.48161339112805</v>
       </c>
       <c r="L148" t="n">
-        <v>38.62826582953539</v>
+        <v>54.27349369645218</v>
       </c>
       <c r="M148" t="n">
         <v>84.76868087165163</v>
@@ -15067,7 +15291,7 @@
         <v>73.75774260644823</v>
       </c>
       <c r="L149" t="n">
-        <v>48.67398235680783</v>
+        <v>52.8265653294479</v>
       </c>
       <c r="M149" t="n">
         <v>85.39700590784228</v>
@@ -15147,7 +15371,7 @@
         <v>86.80051854147119</v>
       </c>
       <c r="L150" t="n">
-        <v>53.97698432564293</v>
+        <v>51.10024026676329</v>
       </c>
       <c r="M150" t="n">
         <v>87.66872650328276</v>
@@ -15225,7 +15449,7 @@
         <v>61.55233094638483</v>
       </c>
       <c r="L151" t="n">
-        <v>46.78005308222387</v>
+        <v>50.22162775827987</v>
       </c>
       <c r="M151" t="n">
         <v>89.24773532795588</v>
@@ -15305,7 +15529,7 @@
         <v>67.0119443764131</v>
       </c>
       <c r="L152" t="n">
-        <v>37.45069776668065</v>
+        <v>49.96921246537399</v>
       </c>
       <c r="M152" t="n">
         <v>90.36785562360491</v>
@@ -15383,7 +15607,7 @@
         <v>80.47715539947613</v>
       </c>
       <c r="L153" t="n">
-        <v>36.85095349639573</v>
+        <v>50.31686236700425</v>
       </c>
       <c r="M153" t="n">
         <v>90.15259557291911</v>
@@ -15463,7 +15687,7 @@
         <v>75.65651402504383</v>
       </c>
       <c r="L154" t="n">
-        <v>32.05299933411636</v>
+        <v>51.57760136614513</v>
       </c>
       <c r="M154" t="n">
         <v>89.30372569807582</v>
@@ -15543,7 +15767,7 @@
         <v>69.52702965016145</v>
       </c>
       <c r="L155" t="n">
-        <v>24.7517647393434</v>
+        <v>52.28944830181403</v>
       </c>
       <c r="M155" t="n">
         <v>88.79409990323373</v>
@@ -15623,7 +15847,7 @@
         <v>73.39867948583843</v>
       </c>
       <c r="L156" t="n">
-        <v>26.73425274389633</v>
+        <v>52.77197229205314</v>
       </c>
       <c r="M156" t="n">
         <v>89.20510718112509</v>
@@ -15703,7 +15927,7 @@
         <v>65.75294010832461</v>
       </c>
       <c r="L157" t="n">
-        <v>20.67017178879324</v>
+        <v>52.88482274734982</v>
       </c>
       <c r="M157" t="n">
         <v>89.62374180480674</v>
@@ -15783,7 +16007,7 @@
         <v>68.37727641547052</v>
       </c>
       <c r="L158" t="n">
-        <v>29.66633584306707</v>
+        <v>52.63581841651992</v>
       </c>
       <c r="M158" t="n">
         <v>89.95735929245305</v>
@@ -15863,7 +16087,7 @@
         <v>75.76030307629998</v>
       </c>
       <c r="L159" t="n">
-        <v>51.66130505982059</v>
+        <v>51.99441298014649</v>
       </c>
       <c r="M159" t="n">
         <v>91.53933219107782</v>
@@ -15943,7 +16167,7 @@
         <v>71.73591559749711</v>
       </c>
       <c r="L160" t="n">
-        <v>53.97032050041754</v>
+        <v>50.97756969656808</v>
       </c>
       <c r="M160" t="n">
         <v>92.69492342774645</v>
@@ -16023,7 +16247,7 @@
         <v>74.03272428885576</v>
       </c>
       <c r="L161" t="n">
-        <v>50.23857837420025</v>
+        <v>49.66637387467503</v>
       </c>
       <c r="M161" t="n">
         <v>91.99718819183596</v>
@@ -16103,7 +16327,7 @@
         <v>79.43796520474839</v>
       </c>
       <c r="L162" t="n">
-        <v>48.83917507686877</v>
+        <v>47.84881136261014</v>
       </c>
       <c r="M162" t="n">
         <v>91.01802175409797</v>
@@ -16183,7 +16407,7 @@
         <v>73.56599768192865</v>
       </c>
       <c r="L163" t="n">
-        <v>46.74007013087154</v>
+        <v>46.42190102768872</v>
       </c>
       <c r="M163" t="n">
         <v>91.137118674737</v>
@@ -16263,7 +16487,7 @@
         <v>67.27540818515132</v>
       </c>
       <c r="L164" t="n">
-        <v>36.27683932313153</v>
+        <v>45.18540199879732</v>
       </c>
       <c r="M164" t="n">
         <v>92.38543931526385</v>
@@ -16343,7 +16567,7 @@
         <v>84.55788525895157</v>
       </c>
       <c r="L165" t="n">
-        <v>35.99695866366523</v>
+        <v>44.22675935917467</v>
       </c>
       <c r="M165" t="n">
         <v>94.02384903400403</v>
@@ -16423,7 +16647,7 @@
         <v>85.06396831123612</v>
       </c>
       <c r="L166" t="n">
-        <v>35.99695866366523</v>
+        <v>43.53165529715432</v>
       </c>
       <c r="M166" t="n">
         <v>92.8584983200618</v>
@@ -16503,7 +16727,7 @@
         <v>83.10959374090689</v>
       </c>
       <c r="L167" t="n">
-        <v>19.80386336597235</v>
+        <v>43.16609640061597</v>
       </c>
       <c r="M167" t="n">
         <v>92.56992824908228</v>
@@ -16583,7 +16807,7 @@
         <v>78.46533817797612</v>
       </c>
       <c r="L168" t="n">
-        <v>26.9085262601168</v>
+        <v>43.11101852506153</v>
       </c>
       <c r="M168" t="n">
         <v>93.22826452664057</v>
@@ -16663,7 +16887,7 @@
         <v>89.04913422558568</v>
       </c>
       <c r="L169" t="n">
-        <v>37.82387197930238</v>
+        <v>43.33191969791464</v>
       </c>
       <c r="M169" t="n">
         <v>93.00248707528647</v>
@@ -16743,7 +16967,7 @@
         <v>85.16514315643664</v>
       </c>
       <c r="L170" t="n">
-        <v>63.01313133126907</v>
+        <v>43.93453482363842</v>
       </c>
       <c r="M170" t="n">
         <v>91.04535038119542</v>
@@ -16823,7 +17047,7 @@
         <v>88.32842195472395</v>
       </c>
       <c r="L171" t="n">
-        <v>63.46293953398276</v>
+        <v>44.47122376294349</v>
       </c>
       <c r="M171" t="n">
         <v>90.88697971861323</v>
@@ -16903,7 +17127,7 @@
         <v>93.38937265718774</v>
       </c>
       <c r="L172" t="n">
-        <v>86.55309393995225</v>
+        <v>45.0474761310949</v>
       </c>
       <c r="M172" t="n">
         <v>94.94428813348</v>
@@ -16983,7 +17207,7 @@
         <v>87.14326254800187</v>
       </c>
       <c r="L173" t="n">
-        <v>104.6053964755284</v>
+        <v>45.58416507039998</v>
       </c>
       <c r="M173" t="n">
         <v>96.16384819295274</v>
@@ -17063,7 +17287,7 @@
         <v>77.25736106159651</v>
       </c>
       <c r="L174" t="n">
-        <v>88.3078027833909</v>
+        <v>45.99351348747959</v>
       </c>
       <c r="M174" t="n">
         <v>96.6674779512479</v>
@@ -20746,7 +20970,7 @@
         </is>
       </c>
       <c r="B182" t="n">
-        <v>88.3078027833909</v>
+        <v>45.99351348747959</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -20766,7 +20990,7 @@
         </is>
       </c>
       <c r="B183" t="n">
-        <v>17.11166706759797</v>
+        <v>55.49644745247897</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -20786,7 +21010,7 @@
         </is>
       </c>
       <c r="B184" t="n">
-        <v>14.90164596214241</v>
+        <v>54.40141454348697</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
@@ -20806,7 +21030,7 @@
         </is>
       </c>
       <c r="B185" t="n">
-        <v>24.58652192668532</v>
+        <v>53.33943935769823</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -20826,7 +21050,7 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>42.34127907782152</v>
+        <v>19.2222394833123</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
@@ -20846,7 +21070,7 @@
         </is>
       </c>
       <c r="B187" t="n">
-        <v>17.21266055694254</v>
+        <v>41.93840028123913</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
@@ -20866,7 +21090,7 @@
         </is>
       </c>
       <c r="B188" t="n">
-        <v>10.78290219283098</v>
+        <v>32.81527198529308</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -20886,7 +21110,7 @@
         </is>
       </c>
       <c r="B189" t="n">
-        <v>22.61658657923002</v>
+        <v>18.38151284855818</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -20906,7 +21130,7 @@
         </is>
       </c>
       <c r="B190" t="n">
-        <v>56.40801157024919</v>
+        <v>70.39177703270168</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -20926,7 +21150,7 @@
         </is>
       </c>
       <c r="B191" t="n">
-        <v>52.98525861247374</v>
+        <v>36.41213164124664</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -20946,7 +21170,7 @@
         </is>
       </c>
       <c r="B192" t="n">
-        <v>40.68240310706825</v>
+        <v>50.17215113891238</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -20966,7 +21190,7 @@
         </is>
       </c>
       <c r="B193" t="n">
-        <v>31.39767831420735</v>
+        <v>51.99413781299535</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -20986,7 +21210,7 @@
         </is>
       </c>
       <c r="B194" t="n">
-        <v>14.64674198252659</v>
+        <v>58.66170336585953</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
@@ -21006,7 +21230,7 @@
         </is>
       </c>
       <c r="B195" t="n">
-        <v>49.97619025586915</v>
+        <v>25.57811725662442</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
@@ -21026,7 +21250,7 @@
         </is>
       </c>
       <c r="B196" t="n">
-        <v>12.59462967598335</v>
+        <v>35.93239717256596</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -21046,7 +21270,7 @@
         </is>
       </c>
       <c r="B197" t="n">
-        <v>17.10411068492214</v>
+        <v>33.13383715500429</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -21066,7 +21290,7 @@
         </is>
       </c>
       <c r="B198" t="n">
-        <v>16.40842691322651</v>
+        <v>34.8524186755283</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
@@ -21086,7 +21310,7 @@
         </is>
       </c>
       <c r="B199" t="n">
-        <v>52.98525861247374</v>
+        <v>34.87942906807599</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -22726,7 +22950,7 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>64.44155391919112</v>
+        <v>64.47410830675643</v>
       </c>
       <c r="C281" t="inlineStr">
         <is>
@@ -23086,7 +23310,7 @@
         </is>
       </c>
       <c r="B299" t="n">
-        <v>37.10332420246828</v>
+        <v>37.13652233571844</v>
       </c>
       <c r="C299" t="inlineStr">
         <is>
@@ -24166,7 +24390,7 @@
         </is>
       </c>
       <c r="B353" t="n">
-        <v>37.62198502689918</v>
+        <v>37.63663830071253</v>
       </c>
       <c r="C353" t="inlineStr">
         <is>
@@ -24526,7 +24750,7 @@
         </is>
       </c>
       <c r="B371" t="n">
-        <v>28.27647006691712</v>
+        <v>28.34741482029767</v>
       </c>
       <c r="C371" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
actualizacion 2 de junio
</commit_message>
<xml_diff>
--- a/results/data/auditoria_normalizacion.xlsx
+++ b/results/data/auditoria_normalizacion.xlsx
@@ -4262,7 +4262,7 @@
         <v>0</v>
       </c>
       <c r="O110" t="n">
-        <v>552.930702666147</v>
+        <v>552.9296809815975</v>
       </c>
       <c r="P110" t="inlineStr"/>
       <c r="Q110" t="inlineStr"/>
@@ -4318,7 +4318,7 @@
         <v>0</v>
       </c>
       <c r="O111" t="n">
-        <v>525.1480962256227</v>
+        <v>525.1496147458497</v>
       </c>
       <c r="P111" t="inlineStr"/>
       <c r="Q111" t="inlineStr"/>
@@ -4376,7 +4376,7 @@
         <v>0</v>
       </c>
       <c r="O112" t="n">
-        <v>493.2286208165917</v>
+        <v>493.2310768572676</v>
       </c>
       <c r="P112" t="inlineStr"/>
       <c r="Q112" t="inlineStr"/>
@@ -4432,7 +4432,7 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>451.3228639758596</v>
+        <v>451.3200727345171</v>
       </c>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr"/>
@@ -4490,7 +4490,7 @@
         <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>481.5500053782423</v>
+        <v>481.5501704967094</v>
       </c>
       <c r="P114" t="inlineStr"/>
       <c r="Q114" t="inlineStr"/>
@@ -4546,7 +4546,7 @@
         <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>383.2677836295125</v>
+        <v>383.2683477409723</v>
       </c>
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr"/>
@@ -4604,7 +4604,7 @@
         <v>0</v>
       </c>
       <c r="O116" t="n">
-        <v>331.104410255819</v>
+        <v>331.1065075457572</v>
       </c>
       <c r="P116" t="inlineStr"/>
       <c r="Q116" t="inlineStr"/>
@@ -4660,7 +4660,7 @@
         <v>0</v>
       </c>
       <c r="O117" t="n">
-        <v>339.1553334257921</v>
+        <v>339.1527258965038</v>
       </c>
       <c r="P117" t="inlineStr"/>
       <c r="Q117" t="inlineStr"/>
@@ -4718,7 +4718,7 @@
         <v>6.617009865593446</v>
       </c>
       <c r="O118" t="n">
-        <v>284.876872648895</v>
+        <v>284.8780679987066</v>
       </c>
       <c r="P118" t="inlineStr"/>
       <c r="Q118" t="inlineStr"/>
@@ -4774,7 +4774,7 @@
         <v>6.552703971541121</v>
       </c>
       <c r="O119" t="n">
-        <v>274.8145676354442</v>
+        <v>274.8140936280106</v>
       </c>
       <c r="P119" t="inlineStr"/>
       <c r="Q119" t="inlineStr"/>
@@ -4832,7 +4832,7 @@
         <v>6.47943270635322</v>
       </c>
       <c r="O120" t="n">
-        <v>270.4139810458742</v>
+        <v>270.415928855229</v>
       </c>
       <c r="P120" t="inlineStr"/>
       <c r="Q120" t="inlineStr"/>
@@ -4888,7 +4888,7 @@
         <v>6.400187311146607</v>
       </c>
       <c r="O121" t="n">
-        <v>227.5793592817693</v>
+        <v>227.5768300005198</v>
       </c>
       <c r="P121" t="inlineStr"/>
       <c r="Q121" t="inlineStr"/>
@@ -4946,7 +4946,7 @@
         <v>6.234925664096019</v>
       </c>
       <c r="O122" t="n">
-        <v>217.551125945396</v>
+        <v>217.5547682473322</v>
       </c>
       <c r="P122" t="inlineStr"/>
       <c r="Q122" t="inlineStr"/>
@@ -5002,7 +5002,7 @@
         <v>6.531064400585945</v>
       </c>
       <c r="O123" t="n">
-        <v>201.696430587921</v>
+        <v>201.6969491571973</v>
       </c>
       <c r="P123" t="inlineStr"/>
       <c r="Q123" t="inlineStr"/>
@@ -5060,7 +5060,7 @@
         <v>6.382259561040986</v>
       </c>
       <c r="O124" t="n">
-        <v>147.3380023709103</v>
+        <v>147.3356997350353</v>
       </c>
       <c r="P124" t="inlineStr"/>
       <c r="Q124" t="inlineStr"/>
@@ -5116,7 +5116,7 @@
         <v>6.417270266653735</v>
       </c>
       <c r="O125" t="n">
-        <v>170.4550206032323</v>
+        <v>170.4525406652386</v>
       </c>
       <c r="P125" t="inlineStr"/>
       <c r="Q125" t="inlineStr"/>
@@ -5176,7 +5176,7 @@
         <v>6.336293698558523</v>
       </c>
       <c r="O126" t="n">
-        <v>156.7014027346077</v>
+        <v>156.7039410505758</v>
       </c>
       <c r="P126" t="inlineStr"/>
       <c r="Q126" t="n">
@@ -5236,7 +5236,7 @@
         <v>6.383028317900934</v>
       </c>
       <c r="O127" t="n">
-        <v>166.3499267852517</v>
+        <v>166.3490695769281</v>
       </c>
       <c r="P127" t="inlineStr"/>
       <c r="Q127" t="n">
@@ -5298,7 +5298,7 @@
         <v>6.456372621653939</v>
       </c>
       <c r="O128" t="n">
-        <v>182.2126002241846</v>
+        <v>182.2160425669692</v>
       </c>
       <c r="P128" t="inlineStr"/>
       <c r="Q128" t="n">
@@ -5358,7 +5358,7 @@
         <v>6.543235690543376</v>
       </c>
       <c r="O129" t="n">
-        <v>198.8480948052696</v>
+        <v>198.8437743663347</v>
       </c>
       <c r="P129" t="inlineStr"/>
       <c r="Q129" t="n">
@@ -5420,7 +5420,7 @@
         <v>6.537509808588505</v>
       </c>
       <c r="O130" t="n">
-        <v>188.4865880891226</v>
+        <v>188.4874594179618</v>
       </c>
       <c r="P130" t="inlineStr"/>
       <c r="Q130" t="n">
@@ -5480,7 +5480,7 @@
         <v>6.488316933693232</v>
       </c>
       <c r="O131" t="n">
-        <v>194.4506144200202</v>
+        <v>194.4496714995352</v>
       </c>
       <c r="P131" t="inlineStr"/>
       <c r="Q131" t="n">
@@ -5542,7 +5542,7 @@
         <v>6.617159603644375</v>
       </c>
       <c r="O132" t="n">
-        <v>216.5383224997886</v>
+        <v>216.5418940274049</v>
       </c>
       <c r="P132" t="inlineStr"/>
       <c r="Q132" t="n">
@@ -5602,7 +5602,7 @@
         <v>6.550681953204485</v>
       </c>
       <c r="O133" t="n">
-        <v>211.3582169747403</v>
+        <v>211.3544504461187</v>
       </c>
       <c r="P133" t="inlineStr"/>
       <c r="Q133" t="n">
@@ -5670,7 +5670,7 @@
         <v>6.626410903450378</v>
       </c>
       <c r="O134" t="n">
-        <v>227.8627519974393</v>
+        <v>227.8648528600462</v>
       </c>
       <c r="P134" t="n">
         <v>425.2998249704278</v>
@@ -5744,7 +5744,7 @@
         <v>6.492051102564349</v>
       </c>
       <c r="O135" t="n">
-        <v>228.7603718571897</v>
+        <v>228.762285784819</v>
       </c>
       <c r="P135" t="n">
         <v>447.708770292318</v>
@@ -5820,7 +5820,7 @@
         <v>6.574321571949497</v>
       </c>
       <c r="O136" t="n">
-        <v>212.4588734889371</v>
+        <v>212.4544059313405</v>
       </c>
       <c r="P136" t="n">
         <v>415.2288435903662</v>
@@ -5894,7 +5894,7 @@
         <v>6.491044392108078</v>
       </c>
       <c r="O137" t="n">
-        <v>239.9688694759318</v>
+        <v>239.9680166596036</v>
       </c>
       <c r="P137" t="n">
         <v>441.0763497510066</v>
@@ -5970,7 +5970,7 @@
         <v>6.723320661239827</v>
       </c>
       <c r="O138" t="n">
-        <v>229.2689746425532</v>
+        <v>229.272147620238</v>
       </c>
       <c r="P138" t="n">
         <v>444.5327589657671</v>
@@ -6048,7 +6048,7 @@
         <v>6.650149818378792</v>
       </c>
       <c r="O139" t="n">
-        <v>239.463196597586</v>
+        <v>239.462611765677</v>
       </c>
       <c r="P139" t="n">
         <v>420.6312828801924</v>
@@ -6128,7 +6128,7 @@
         <v>6.710086103433602</v>
       </c>
       <c r="O140" t="n">
-        <v>264.1658008926404</v>
+        <v>264.1619106148757</v>
       </c>
       <c r="P140" t="n">
         <v>461.7985807858078</v>
@@ -6206,7 +6206,7 @@
         <v>6.765520024431838</v>
       </c>
       <c r="O141" t="n">
-        <v>237.5213686242965</v>
+        <v>237.5269824845462</v>
       </c>
       <c r="P141" t="n">
         <v>422.1850788246194</v>
@@ -6286,7 +6286,7 @@
         <v>6.959267096137754</v>
       </c>
       <c r="O142" t="n">
-        <v>253.7185619782126</v>
+        <v>253.7230816692874</v>
       </c>
       <c r="P142" t="n">
         <v>425.6576300924954</v>
@@ -6364,7 +6364,7 @@
         <v>7.087489455717128</v>
       </c>
       <c r="O143" t="n">
-        <v>255.4061665187805</v>
+        <v>255.3965172841019</v>
       </c>
       <c r="P143" t="n">
         <v>433.0122881080762</v>
@@ -6444,7 +6444,7 @@
         <v>6.813274287459069</v>
       </c>
       <c r="O144" t="n">
-        <v>299.5413867609174</v>
+        <v>299.5412156647211</v>
       </c>
       <c r="P144" t="n">
         <v>405.7070181491501</v>
@@ -6522,7 +6522,7 @@
         <v>6.755777513953618</v>
       </c>
       <c r="O145" t="n">
-        <v>263.2712336362275</v>
+        <v>263.2875819407082</v>
       </c>
       <c r="P145" t="n">
         <v>381.7595628392513</v>
@@ -6602,7 +6602,7 @@
         <v>6.654600181971241</v>
       </c>
       <c r="O146" t="n">
-        <v>275.3914833868785</v>
+        <v>275.3953649846974</v>
       </c>
       <c r="P146" t="n">
         <v>366.5992167587976</v>
@@ -6680,7 +6680,7 @@
         <v>6.765157684348584</v>
       </c>
       <c r="O147" t="n">
-        <v>290.1582515347931</v>
+        <v>290.1232551604963</v>
       </c>
       <c r="P147" t="n">
         <v>537.8893473769159</v>
@@ -6760,7 +6760,7 @@
         <v>6.58154487084704</v>
       </c>
       <c r="O148" t="n">
-        <v>258.8348425073008</v>
+        <v>258.854111555052</v>
       </c>
       <c r="P148" t="n">
         <v>585.3072291100987</v>
@@ -6838,7 +6838,7 @@
         <v>6.527120675067359</v>
       </c>
       <c r="O149" t="n">
-        <v>276.5909650425576</v>
+        <v>276.6067966294875</v>
       </c>
       <c r="P149" t="n">
         <v>712.1799440722901</v>
@@ -6918,7 +6918,7 @@
         <v>5.472470537385679</v>
       </c>
       <c r="O150" t="n">
-        <v>299.2403494773894</v>
+        <v>299.2282084729392</v>
       </c>
       <c r="P150" t="n">
         <v>761.6192751927493</v>
@@ -6996,7 +6996,7 @@
         <v>1.479982759352952</v>
       </c>
       <c r="O151" t="n">
-        <v>221.5034183491462</v>
+        <v>221.5271784842887</v>
       </c>
       <c r="P151" t="n">
         <v>1096.997455120887</v>
@@ -7076,7 +7076,7 @@
         <v>4.083082488224957</v>
       </c>
       <c r="O152" t="n">
-        <v>228.8289567622929</v>
+        <v>228.8584744136809</v>
       </c>
       <c r="P152" t="n">
         <v>744.9286298465894</v>
@@ -7154,7 +7154,7 @@
         <v>3.280692157242492</v>
       </c>
       <c r="O153" t="n">
-        <v>251.7354113988364</v>
+        <v>251.7195207021782</v>
       </c>
       <c r="P153" t="n">
         <v>666.970147803431</v>
@@ -7234,7 +7234,7 @@
         <v>3.426329398904774</v>
       </c>
       <c r="O154" t="n">
-        <v>290.7867870782546</v>
+        <v>290.7212526032689</v>
       </c>
       <c r="P154" t="n">
         <v>692.9025170546591</v>
@@ -7314,7 +7314,7 @@
         <v>4.165414177269469</v>
       </c>
       <c r="O155" t="n">
-        <v>323.6775355952332</v>
+        <v>323.7462097791511</v>
       </c>
       <c r="P155" t="n">
         <v>338.8360557706577</v>
@@ -7394,7 +7394,7 @@
         <v>4.786973259298917</v>
       </c>
       <c r="O156" t="n">
-        <v>343.363727708272</v>
+        <v>343.236628865448</v>
       </c>
       <c r="P156" t="n">
         <v>541.049221057197</v>
@@ -7474,7 +7474,7 @@
         <v>4.976827111661795</v>
       </c>
       <c r="O157" t="n">
-        <v>334.6788494907451</v>
+        <v>334.2363118337353</v>
       </c>
       <c r="P157" t="n">
         <v>693.069746725972</v>
@@ -7554,7 +7554,7 @@
         <v>5.192273742736051</v>
       </c>
       <c r="O158" t="n">
-        <v>351.3720063040757</v>
+        <v>351.4135012046711</v>
       </c>
       <c r="P158" t="n">
         <v>1377.512034330812</v>
@@ -7634,7 +7634,7 @@
         <v>5.735647502856111</v>
       </c>
       <c r="O159" t="n">
-        <v>326.4146640868744</v>
+        <v>327.8869497430796</v>
       </c>
       <c r="P159" t="n">
         <v>1418.313584103855</v>
@@ -7714,7 +7714,7 @@
         <v>5.654112693519551</v>
       </c>
       <c r="O160" t="n">
-        <v>335.363456463086</v>
+        <v>334.6309243564401</v>
       </c>
       <c r="P160" t="n">
         <v>1244.637557697542</v>
@@ -7794,7 +7794,7 @@
         <v>5.854283795452693</v>
       </c>
       <c r="O161" t="n">
-        <v>339.6848078506592</v>
+        <v>338.9415742901182</v>
       </c>
       <c r="P161" t="n">
         <v>1131.605035198721</v>
@@ -7874,7 +7874,7 @@
         <v>6.315976867964248</v>
       </c>
       <c r="O162" t="n">
-        <v>322.3791073011038</v>
+        <v>322.4443039877935</v>
       </c>
       <c r="P162" t="n">
         <v>456.7108368970343</v>
@@ -7954,7 +7954,7 @@
         <v>6.525818118040934</v>
       </c>
       <c r="O163" t="n">
-        <v>291.7694096348481</v>
+        <v>293.4619211322573</v>
       </c>
       <c r="P163" t="n">
         <v>425.6131793057602</v>
@@ -8034,7 +8034,7 @@
         <v>6.677721800337137</v>
       </c>
       <c r="O164" t="n">
-        <v>261.5557444225678</v>
+        <v>260.4625011949565</v>
       </c>
       <c r="P164" t="n">
         <v>489.0302385593588</v>
@@ -8114,7 +8114,7 @@
         <v>6.965183001091694</v>
       </c>
       <c r="O165" t="n">
-        <v>262.4945374175591</v>
+        <v>261.159331130176</v>
       </c>
       <c r="P165" t="n">
         <v>495.3304753337681</v>
@@ -8194,7 +8194,7 @@
         <v>7.189593813264385</v>
       </c>
       <c r="O166" t="n">
-        <v>259.0228140830272</v>
+        <v>260.2465249374989</v>
       </c>
       <c r="P166" t="n">
         <v>621.7168389017788</v>
@@ -8274,7 +8274,7 @@
         <v>7.227650679904569</v>
       </c>
       <c r="O167" t="n">
-        <v>287.1753585094702</v>
+        <v>288.9767907350401</v>
       </c>
       <c r="P167" t="n">
         <v>735.7304942162914</v>
@@ -8354,7 +8354,7 @@
         <v>7.396530534393766</v>
       </c>
       <c r="O168" t="n">
-        <v>316.4440925179414</v>
+        <v>314.864816447407</v>
       </c>
       <c r="P168" t="n">
         <v>590.3012052055421</v>
@@ -8434,7 +8434,7 @@
         <v>7.477067434560478</v>
       </c>
       <c r="O169" t="n">
-        <v>336.6109786452491</v>
+        <v>334.4015332964078</v>
       </c>
       <c r="P169" t="n">
         <v>798.0687288374654</v>
@@ -8514,7 +8514,7 @@
         <v>7.704817404130716</v>
       </c>
       <c r="O170" t="n">
-        <v>334.5339366157513</v>
+        <v>337.8684093157943</v>
       </c>
       <c r="P170" t="n">
         <v>745.7487044199559</v>
@@ -8594,7 +8594,7 @@
         <v>7.360529111064243</v>
       </c>
       <c r="O171" t="n">
-        <v>345.7829207119789</v>
+        <v>347.6919135602138</v>
       </c>
       <c r="P171" t="n">
         <v>772.7461062814623</v>
@@ -8674,7 +8674,7 @@
         <v>7.765590025928953</v>
       </c>
       <c r="O172" t="n">
-        <v>355.6478371569374</v>
+        <v>353.5087667467222</v>
       </c>
       <c r="P172" t="n">
         <v>1140.100345143426</v>
@@ -8754,7 +8754,7 @@
         <v>7.855907089254644</v>
       </c>
       <c r="O173" t="n">
-        <v>373.2577707685841</v>
+        <v>370.1805582592172</v>
       </c>
       <c r="P173" t="n">
         <v>1047.901579369782</v>
@@ -8834,7 +8834,7 @@
         <v>7.942472463187705</v>
       </c>
       <c r="O174" t="n">
-        <v>252.653161186876</v>
+        <v>373.0712128332248</v>
       </c>
       <c r="P174" t="n">
         <v>975.8073104306128</v>
@@ -12838,7 +12838,7 @@
         <v>0</v>
       </c>
       <c r="O112" t="n">
-        <v>120</v>
+        <v>113.8443909981209</v>
       </c>
       <c r="P112" t="inlineStr"/>
       <c r="Q112" t="inlineStr"/>
@@ -12894,7 +12894,7 @@
         <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>120</v>
+        <v>104.1707654616363</v>
       </c>
       <c r="P113" t="inlineStr"/>
       <c r="Q113" t="inlineStr"/>
@@ -12952,7 +12952,7 @@
         <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>120</v>
+        <v>111.1482801216592</v>
       </c>
       <c r="P114" t="inlineStr"/>
       <c r="Q114" t="inlineStr"/>
@@ -13008,7 +13008,7 @@
         <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>120</v>
+        <v>88.46350865692438</v>
       </c>
       <c r="P115" t="inlineStr"/>
       <c r="Q115" t="inlineStr"/>
@@ -13066,7 +13066,7 @@
         <v>0</v>
       </c>
       <c r="O116" t="n">
-        <v>120</v>
+        <v>76.42385177195479</v>
       </c>
       <c r="P116" t="inlineStr"/>
       <c r="Q116" t="inlineStr"/>
@@ -13122,7 +13122,7 @@
         <v>0</v>
       </c>
       <c r="O117" t="n">
-        <v>120</v>
+        <v>78.2810275886435</v>
       </c>
       <c r="P117" t="inlineStr"/>
       <c r="Q117" t="inlineStr"/>
@@ -13180,7 +13180,7 @@
         <v>26.7128482831499</v>
       </c>
       <c r="O118" t="n">
-        <v>106.8039863563101</v>
+        <v>65.75370385556468</v>
       </c>
       <c r="P118" t="inlineStr"/>
       <c r="Q118" t="inlineStr"/>
@@ -13236,7 +13236,7 @@
         <v>26.45324558851526</v>
       </c>
       <c r="O119" t="n">
-        <v>103.0314993959728</v>
+        <v>63.43080271042022</v>
       </c>
       <c r="P119" t="inlineStr"/>
       <c r="Q119" t="inlineStr"/>
@@ -13294,7 +13294,7 @@
         <v>26.15744971844165</v>
       </c>
       <c r="O120" t="n">
-        <v>101.3816631502223</v>
+        <v>62.41564690706517</v>
       </c>
       <c r="P120" t="inlineStr"/>
       <c r="Q120" t="inlineStr"/>
@@ -13350,7 +13350,7 @@
         <v>25.83753630403077</v>
       </c>
       <c r="O121" t="n">
-        <v>85.32241511112417</v>
+        <v>52.52780457746683</v>
       </c>
       <c r="P121" t="inlineStr"/>
       <c r="Q121" t="inlineStr"/>
@@ -13408,7 +13408,7 @@
         <v>25.17037554798588</v>
       </c>
       <c r="O122" t="n">
-        <v>81.56270205868569</v>
+        <v>50.21457743025003</v>
       </c>
       <c r="P122" t="inlineStr"/>
       <c r="Q122" t="inlineStr"/>
@@ -13464,7 +13464,7 @@
         <v>26.36588670775496</v>
       </c>
       <c r="O123" t="n">
-        <v>75.61857380812661</v>
+        <v>46.55437870883571</v>
       </c>
       <c r="P123" t="inlineStr"/>
       <c r="Q123" t="inlineStr"/>
@@ -13522,7 +13522,7 @@
         <v>25.7651620325158</v>
       </c>
       <c r="O124" t="n">
-        <v>55.23890320989076</v>
+        <v>34.00706848297602</v>
       </c>
       <c r="P124" t="inlineStr"/>
       <c r="Q124" t="inlineStr"/>
@@ -13578,7 +13578,7 @@
         <v>25.9065001423745</v>
       </c>
       <c r="O125" t="n">
-        <v>63.90576927355495</v>
+        <v>39.3427474395171</v>
       </c>
       <c r="P125" t="inlineStr"/>
       <c r="Q125" t="inlineStr"/>
@@ -13638,7 +13638,7 @@
         <v>25.57959798838723</v>
       </c>
       <c r="O126" t="n">
-        <v>58.74936187013285</v>
+        <v>36.16938504682012</v>
       </c>
       <c r="P126" t="inlineStr"/>
       <c r="Q126" t="n">
@@ -13698,7 +13698,7 @@
         <v>25.7682655015726</v>
       </c>
       <c r="O127" t="n">
-        <v>62.36671705057108</v>
+        <v>38.39561091680711</v>
       </c>
       <c r="P127" t="inlineStr"/>
       <c r="Q127" t="n">
@@ -13760,7 +13760,7 @@
         <v>26.06435622810677</v>
       </c>
       <c r="O128" t="n">
-        <v>68.31383638599867</v>
+        <v>42.05792248189446</v>
       </c>
       <c r="P128" t="inlineStr"/>
       <c r="Q128" t="n">
@@ -13820,7 +13820,7 @@
         <v>26.41502216752414</v>
       </c>
       <c r="O129" t="n">
-        <v>74.55069626075047</v>
+        <v>45.89582745017092</v>
       </c>
       <c r="P129" t="inlineStr"/>
       <c r="Q129" t="n">
@@ -13882,7 +13882,7 @@
         <v>26.39190679984983</v>
       </c>
       <c r="O130" t="n">
-        <v>70.66603475189535</v>
+        <v>43.5054501531957</v>
       </c>
       <c r="P130" t="inlineStr"/>
       <c r="Q130" t="n">
@@ -13942,7 +13942,7 @@
         <v>26.19331531662986</v>
       </c>
       <c r="O131" t="n">
-        <v>72.90202457076327</v>
+        <v>44.88160918955095</v>
       </c>
       <c r="P131" t="inlineStr"/>
       <c r="Q131" t="n">
@@ -14004,7 +14004,7 @@
         <v>26.7134527751966</v>
       </c>
       <c r="O132" t="n">
-        <v>81.18298908170566</v>
+        <v>49.98079238681758</v>
       </c>
       <c r="P132" t="inlineStr"/>
       <c r="Q132" t="n">
@@ -14064,7 +14064,7 @@
         <v>26.44508270676815</v>
       </c>
       <c r="O133" t="n">
-        <v>79.24090120817236</v>
+        <v>48.7834603794519</v>
       </c>
       <c r="P133" t="inlineStr"/>
       <c r="Q133" t="n">
@@ -14120,7 +14120,7 @@
         <v>42.42070093811161</v>
       </c>
       <c r="K134" t="n">
-        <v>82.70112145333562</v>
+        <v>17.29887854666439</v>
       </c>
       <c r="L134" t="n">
         <v>65.2257522279661</v>
@@ -14132,7 +14132,7 @@
         <v>26.75080024379033</v>
       </c>
       <c r="O134" t="n">
-        <v>85.42866266802994</v>
+        <v>52.59428414166064</v>
       </c>
       <c r="P134" t="n">
         <v>3.21009247639399</v>
@@ -14194,7 +14194,7 @@
         <v>43.28396680470292</v>
       </c>
       <c r="K135" t="n">
-        <v>81.1952384155465</v>
+        <v>18.8047615844535</v>
       </c>
       <c r="L135" t="n">
         <v>65.27035296816766</v>
@@ -14206,7 +14206,7 @@
         <v>26.20839014476885</v>
       </c>
       <c r="O135" t="n">
-        <v>85.76519184417016</v>
+        <v>52.80142377575143</v>
       </c>
       <c r="P135" t="n">
         <v>3.379231475655806</v>
@@ -14270,7 +14270,7 @@
         <v>42.36692923076075</v>
       </c>
       <c r="K136" t="n">
-        <v>94.01172820054809</v>
+        <v>5.988271799451905</v>
       </c>
       <c r="L136" t="n">
         <v>65.31950415889682</v>
@@ -14282,7 +14282,7 @@
         <v>26.54051577424634</v>
       </c>
       <c r="O136" t="n">
-        <v>79.65355142520188</v>
+        <v>49.03734495448317</v>
       </c>
       <c r="P136" t="n">
         <v>3.134078380784409</v>
@@ -14344,7 +14344,7 @@
         <v>39.19088298880057</v>
       </c>
       <c r="K137" t="n">
-        <v>79.22487677648353</v>
+        <v>20.77512322351647</v>
       </c>
       <c r="L137" t="n">
         <v>65.34147454758342</v>
@@ -14356,7 +14356,7 @@
         <v>26.20432605778248</v>
       </c>
       <c r="O137" t="n">
-        <v>89.96740108501042</v>
+        <v>55.38785773538181</v>
       </c>
       <c r="P137" t="n">
         <v>3.329171066434088</v>
@@ -14420,7 +14420,7 @@
         <v>39.96676239466897</v>
       </c>
       <c r="K138" t="n">
-        <v>78.82165728669344</v>
+        <v>21.17834271330656</v>
       </c>
       <c r="L138" t="n">
         <v>65.43988489863935</v>
@@ -14432,7 +14432,7 @@
         <v>27.14202463510446</v>
       </c>
       <c r="O138" t="n">
-        <v>85.95587353919036</v>
+        <v>52.91910677033545</v>
       </c>
       <c r="P138" t="n">
         <v>3.355259469401131</v>
@@ -14498,7 +14498,7 @@
         <v>37.46496578797295</v>
       </c>
       <c r="K139" t="n">
-        <v>87.74035427029538</v>
+        <v>12.25964572970462</v>
       </c>
       <c r="L139" t="n">
         <v>65.09088735351374</v>
@@ -14510,7 +14510,7 @@
         <v>26.84663416965263</v>
       </c>
       <c r="O139" t="n">
-        <v>89.77781784963786</v>
+        <v>55.2712034630615</v>
       </c>
       <c r="P139" t="n">
         <v>3.174855095704648</v>
@@ -14578,7 +14578,7 @@
         <v>37.66954596759271</v>
       </c>
       <c r="K140" t="n">
-        <v>80.9086771312366</v>
+        <v>19.0913228687634</v>
       </c>
       <c r="L140" t="n">
         <v>64.39979421539816</v>
@@ -14590,7 +14590,7 @@
         <v>27.0885967663309</v>
       </c>
       <c r="O140" t="n">
-        <v>99.03914042581626</v>
+        <v>60.97213506997507</v>
       </c>
       <c r="P140" t="n">
         <v>3.485579026262284</v>
@@ -14656,7 +14656,7 @@
         <v>38.80948114742625</v>
       </c>
       <c r="K141" t="n">
-        <v>73.95337161673879</v>
+        <v>26.0466283832612</v>
       </c>
       <c r="L141" t="n">
         <v>63.37641266648133</v>
@@ -14668,7 +14668,7 @@
         <v>27.31238333329157</v>
       </c>
       <c r="O141" t="n">
-        <v>89.04980168448874</v>
+        <v>54.82443409460941</v>
       </c>
       <c r="P141" t="n">
         <v>3.186582889553148</v>
@@ -14736,7 +14736,7 @@
         <v>39.14351499047054</v>
       </c>
       <c r="K142" t="n">
-        <v>76.089567400549</v>
+        <v>23.91043259945099</v>
       </c>
       <c r="L142" t="n">
         <v>61.87316569812717</v>
@@ -14748,7 +14748,7 @@
         <v>28.09453966022951</v>
       </c>
       <c r="O142" t="n">
-        <v>95.1223368183403</v>
+        <v>58.56271242853036</v>
       </c>
       <c r="P142" t="n">
         <v>3.212793130057424</v>
@@ -14814,7 +14814,7 @@
         <v>41.55696002520011</v>
       </c>
       <c r="K143" t="n">
-        <v>89.02145000630114</v>
+        <v>10.97854999369886</v>
       </c>
       <c r="L143" t="n">
         <v>60.54802105380879</v>
@@ -14826,7 +14826,7 @@
         <v>28.61217292775133</v>
       </c>
       <c r="O143" t="n">
-        <v>95.75504136416633</v>
+        <v>58.94896395926725</v>
       </c>
       <c r="P143" t="n">
         <v>3.268304867838901</v>
@@ -14894,7 +14894,7 @@
         <v>39.39736777797776</v>
       </c>
       <c r="K144" t="n">
-        <v>79.94236487697448</v>
+        <v>20.05763512302552</v>
       </c>
       <c r="L144" t="n">
         <v>59.26388088669739</v>
@@ -14906,7 +14906,7 @@
         <v>27.5051671448668</v>
       </c>
       <c r="O144" t="n">
-        <v>112.301900422057</v>
+        <v>69.1381562846155</v>
       </c>
       <c r="P144" t="n">
         <v>3.062209223037848</v>
@@ -14972,7 +14972,7 @@
         <v>40.07713022471152</v>
       </c>
       <c r="K145" t="n">
-        <v>85.0210250476506</v>
+        <v>14.97897495234941</v>
       </c>
       <c r="L145" t="n">
         <v>58.05006117234873</v>
@@ -14984,7 +14984,7 @@
         <v>27.27305284873919</v>
       </c>
       <c r="O145" t="n">
-        <v>98.70375570974463</v>
+        <v>60.77032820882388</v>
       </c>
       <c r="P145" t="n">
         <v>2.88145780578901</v>
@@ -15052,7 +15052,7 @@
         <v>40.12258953784664</v>
       </c>
       <c r="K146" t="n">
-        <v>82.30011772239232</v>
+        <v>17.69988227760768</v>
       </c>
       <c r="L146" t="n">
         <v>56.94285208470484</v>
@@ -15064,7 +15064,7 @@
         <v>26.86460027365802</v>
       </c>
       <c r="O146" t="n">
-        <v>103.2477924964691</v>
+        <v>63.5649679865182</v>
       </c>
       <c r="P146" t="n">
         <v>2.767030030287863</v>
@@ -15130,7 +15130,7 @@
         <v>37.71954073672836</v>
       </c>
       <c r="K147" t="n">
-        <v>80.84945909815104</v>
+        <v>19.15054090184896</v>
       </c>
       <c r="L147" t="n">
         <v>55.67209997652607</v>
@@ -15142,7 +15142,7 @@
         <v>27.31092056750045</v>
       </c>
       <c r="O147" t="n">
-        <v>108.7840429092587</v>
+        <v>66.96436386083015</v>
       </c>
       <c r="P147" t="n">
         <v>4.059899500939534</v>
@@ -15210,7 +15210,7 @@
         <v>38.39617730254001</v>
       </c>
       <c r="K148" t="n">
-        <v>96.48161339112805</v>
+        <v>3.518386608871948</v>
       </c>
       <c r="L148" t="n">
         <v>54.27349369645218</v>
@@ -15222,7 +15222,7 @@
         <v>26.56967620946908</v>
       </c>
       <c r="O148" t="n">
-        <v>97.04049588384393</v>
+        <v>59.74702339340306</v>
       </c>
       <c r="P148" t="n">
         <v>4.417801800590877</v>
@@ -15288,7 +15288,7 @@
         <v>38.76897377179843</v>
       </c>
       <c r="K149" t="n">
-        <v>73.75774260644823</v>
+        <v>26.24225739355177</v>
       </c>
       <c r="L149" t="n">
         <v>52.8265653294479</v>
@@ -15300,7 +15300,7 @@
         <v>26.34996590008077</v>
       </c>
       <c r="O149" t="n">
-        <v>103.6974935241327</v>
+        <v>63.8445827640698</v>
       </c>
       <c r="P149" t="n">
         <v>5.375415991445831</v>
@@ -15368,7 +15368,7 @@
         <v>33.47182996908115</v>
       </c>
       <c r="K150" t="n">
-        <v>86.80051854147119</v>
+        <v>13.1994814585288</v>
       </c>
       <c r="L150" t="n">
         <v>51.10024026676329</v>
@@ -15380,7 +15380,7 @@
         <v>22.0923465686991</v>
       </c>
       <c r="O150" t="n">
-        <v>112.1890376907875</v>
+        <v>69.06590999925676</v>
       </c>
       <c r="P150" t="n">
         <v>5.748575855498849</v>
@@ -15446,7 +15446,7 @@
         <v>19.51275266953165</v>
       </c>
       <c r="K151" t="n">
-        <v>61.55233094638483</v>
+        <v>38.44766905361517</v>
       </c>
       <c r="L151" t="n">
         <v>50.22162775827987</v>
@@ -15458,7 +15458,7 @@
         <v>5.974685804511385</v>
       </c>
       <c r="O151" t="n">
-        <v>83.04446707541464</v>
+        <v>51.13146333918858</v>
       </c>
       <c r="P151" t="n">
         <v>8.279954682680076</v>
@@ -15526,7 +15526,7 @@
         <v>42.02935885401434</v>
       </c>
       <c r="K152" t="n">
-        <v>67.0119443764131</v>
+        <v>32.9880556235869</v>
       </c>
       <c r="L152" t="n">
         <v>49.96921246537399</v>
@@ -15538,7 +15538,7 @@
         <v>16.48339132795859</v>
       </c>
       <c r="O152" t="n">
-        <v>85.79090520307072</v>
+        <v>52.82362540980803</v>
       </c>
       <c r="P152" t="n">
         <v>5.622597635179587</v>
@@ -15604,7 +15604,7 @@
         <v>40.4659788953466</v>
       </c>
       <c r="K153" t="n">
-        <v>80.47715539947613</v>
+        <v>19.52284460052387</v>
       </c>
       <c r="L153" t="n">
         <v>50.31686236700425</v>
@@ -15616,7 +15616,7 @@
         <v>13.24414405301461</v>
       </c>
       <c r="O153" t="n">
-        <v>94.37882827918538</v>
+        <v>58.10026350989877</v>
       </c>
       <c r="P153" t="n">
         <v>5.034179954322936</v>
@@ -15684,7 +15684,7 @@
         <v>42.67529602187258</v>
       </c>
       <c r="K154" t="n">
-        <v>75.65651402504383</v>
+        <v>24.34348597495617</v>
       </c>
       <c r="L154" t="n">
         <v>51.57760136614513</v>
@@ -15696,7 +15696,7 @@
         <v>13.83208114543605</v>
       </c>
       <c r="O154" t="n">
-        <v>109.0196889305876</v>
+        <v>67.10238974339346</v>
       </c>
       <c r="P154" t="n">
         <v>5.229913172492557</v>
@@ -15764,7 +15764,7 @@
         <v>45.21542048452616</v>
       </c>
       <c r="K155" t="n">
-        <v>69.52702965016145</v>
+        <v>30.47297034983855</v>
       </c>
       <c r="L155" t="n">
         <v>52.28944830181403</v>
@@ -15776,7 +15776,7 @@
         <v>16.81576410101086</v>
       </c>
       <c r="O155" t="n">
-        <v>120</v>
+        <v>74.72499568579096</v>
       </c>
       <c r="P155" t="n">
         <v>2.557478300011133</v>
@@ -15844,7 +15844,7 @@
         <v>42.05292043064004</v>
       </c>
       <c r="K156" t="n">
-        <v>73.39867948583843</v>
+        <v>26.60132051416157</v>
       </c>
       <c r="L156" t="n">
         <v>52.77197229205314</v>
@@ -15856,7 +15856,7 @@
         <v>19.32499618536978</v>
       </c>
       <c r="O156" t="n">
-        <v>120</v>
+        <v>79.22364752524051</v>
       </c>
       <c r="P156" t="n">
         <v>4.083749702919116</v>
@@ -15924,7 +15924,7 @@
         <v>43.54944199106242</v>
       </c>
       <c r="K157" t="n">
-        <v>65.75294010832461</v>
+        <v>34.24705989167539</v>
       </c>
       <c r="L157" t="n">
         <v>52.88482274734982</v>
@@ -15936,7 +15936,7 @@
         <v>20.09143559790741</v>
       </c>
       <c r="O157" t="n">
-        <v>120</v>
+        <v>77.14625285296228</v>
       </c>
       <c r="P157" t="n">
         <v>5.231175394290434</v>
@@ -16004,7 +16004,7 @@
         <v>42.72232205336867</v>
       </c>
       <c r="K158" t="n">
-        <v>68.37727641547052</v>
+        <v>31.62272358452948</v>
       </c>
       <c r="L158" t="n">
         <v>52.63581841651992</v>
@@ -16016,7 +16016,7 @@
         <v>20.96119297864334</v>
       </c>
       <c r="O158" t="n">
-        <v>120</v>
+        <v>81.11098004625605</v>
       </c>
       <c r="P158" t="n">
         <v>10.39723215934779</v>
@@ -16084,7 +16084,7 @@
         <v>40.85049531208663</v>
       </c>
       <c r="K159" t="n">
-        <v>75.76030307629998</v>
+        <v>24.23969692370003</v>
       </c>
       <c r="L159" t="n">
         <v>51.99441298014649</v>
@@ -16096,7 +16096,7 @@
         <v>23.15479116120099</v>
       </c>
       <c r="O159" t="n">
-        <v>120</v>
+        <v>75.68073436811133</v>
       </c>
       <c r="P159" t="n">
         <v>10.70519548371729</v>
@@ -16164,7 +16164,7 @@
         <v>42.28464178177644</v>
       </c>
       <c r="K160" t="n">
-        <v>71.73591559749711</v>
+        <v>28.26408440250289</v>
       </c>
       <c r="L160" t="n">
         <v>50.97756969656808</v>
@@ -16176,7 +16176,7 @@
         <v>22.8256353890556</v>
       </c>
       <c r="O160" t="n">
-        <v>120</v>
+        <v>77.23733475034352</v>
       </c>
       <c r="P160" t="n">
         <v>9.39431766773024</v>
@@ -16244,7 +16244,7 @@
         <v>43.12882438476942</v>
       </c>
       <c r="K161" t="n">
-        <v>74.03272428885576</v>
+        <v>25.96727571114423</v>
       </c>
       <c r="L161" t="n">
         <v>49.66637387467503</v>
@@ -16256,7 +16256,7 @@
         <v>23.63372550607576</v>
       </c>
       <c r="O161" t="n">
-        <v>120</v>
+        <v>78.23229094741154</v>
       </c>
       <c r="P161" t="n">
         <v>8.541166952028611</v>
@@ -16324,7 +16324,7 @@
         <v>48.69723915772703</v>
       </c>
       <c r="K162" t="n">
-        <v>79.43796520474839</v>
+        <v>20.56203479525161</v>
       </c>
       <c r="L162" t="n">
         <v>47.84881136261014</v>
@@ -16336,7 +16336,7 @@
         <v>25.4975790063571</v>
       </c>
       <c r="O162" t="n">
-        <v>120</v>
+        <v>74.42449825383997</v>
       </c>
       <c r="P162" t="n">
         <v>3.447177579987748</v>
@@ -16404,7 +16404,7 @@
         <v>48.2079363206068</v>
       </c>
       <c r="K163" t="n">
-        <v>73.56599768192865</v>
+        <v>26.43400231807135</v>
       </c>
       <c r="L163" t="n">
         <v>46.42190102768872</v>
@@ -16416,7 +16416,7 @@
         <v>26.34470748140922</v>
       </c>
       <c r="O163" t="n">
-        <v>109.3880867059211</v>
+        <v>67.73497303801965</v>
       </c>
       <c r="P163" t="n">
         <v>3.212457622898261</v>
@@ -16484,7 +16484,7 @@
         <v>45.51583536110695</v>
       </c>
       <c r="K164" t="n">
-        <v>67.27540818515132</v>
+        <v>32.72459181484868</v>
       </c>
       <c r="L164" t="n">
         <v>45.18540199879732</v>
@@ -16496,7 +16496,7 @@
         <v>26.95794217521398</v>
       </c>
       <c r="O164" t="n">
-        <v>98.06059684301584</v>
+        <v>60.11826143503116</v>
       </c>
       <c r="P164" t="n">
         <v>3.691119058508219</v>
@@ -16564,7 +16564,7 @@
         <v>45.4378970506257</v>
       </c>
       <c r="K165" t="n">
-        <v>84.55788525895157</v>
+        <v>15.44211474104843</v>
       </c>
       <c r="L165" t="n">
         <v>44.22675935917467</v>
@@ -16576,7 +16576,7 @@
         <v>28.11842215016108</v>
       </c>
       <c r="O165" t="n">
-        <v>98.41256235462836</v>
+        <v>60.27909919105782</v>
       </c>
       <c r="P165" t="n">
         <v>3.738672199801982</v>
@@ -16644,7 +16644,7 @@
         <v>47.10675996785778</v>
       </c>
       <c r="K166" t="n">
-        <v>85.06396831123612</v>
+        <v>14.93603168876387</v>
       </c>
       <c r="L166" t="n">
         <v>43.53165529715432</v>
@@ -16656,7 +16656,7 @@
         <v>29.02436790215973</v>
       </c>
       <c r="O166" t="n">
-        <v>97.1109688338682</v>
+        <v>60.06841119920058</v>
       </c>
       <c r="P166" t="n">
         <v>4.692615491071093</v>
@@ -16724,7 +16724,7 @@
         <v>46.86404277307435</v>
       </c>
       <c r="K167" t="n">
-        <v>83.10959374090689</v>
+        <v>16.89040625909312</v>
       </c>
       <c r="L167" t="n">
         <v>43.16609640061597</v>
@@ -16736,7 +16736,7 @@
         <v>29.17800335462858</v>
       </c>
       <c r="O167" t="n">
-        <v>107.6657181290946</v>
+        <v>66.69974439453719</v>
       </c>
       <c r="P167" t="n">
         <v>5.553171634391263</v>
@@ -16804,7 +16804,7 @@
         <v>50.67928664850857</v>
       </c>
       <c r="K168" t="n">
-        <v>78.46533817797612</v>
+        <v>21.53466182202388</v>
       </c>
       <c r="L168" t="n">
         <v>43.11101852506153</v>
@@ -16816,7 +16816,7 @@
         <v>29.85977080286946</v>
       </c>
       <c r="O168" t="n">
-        <v>118.6389411873243</v>
+        <v>72.67505020889683</v>
       </c>
       <c r="P168" t="n">
         <v>4.455495503127409</v>
@@ -16884,7 +16884,7 @@
         <v>50.46898886018264</v>
       </c>
       <c r="K169" t="n">
-        <v>89.04913422558568</v>
+        <v>10.95086577441433</v>
       </c>
       <c r="L169" t="n">
         <v>43.33191969791464</v>
@@ -16896,7 +16896,7 @@
         <v>30.18489801879444</v>
       </c>
       <c r="O169" t="n">
-        <v>120</v>
+        <v>77.18438819698321</v>
       </c>
       <c r="P169" t="n">
         <v>6.023690280767448</v>
@@ -16964,7 +16964,7 @@
         <v>43.0945382539754</v>
       </c>
       <c r="K170" t="n">
-        <v>85.16514315643664</v>
+        <v>14.83485684356336</v>
       </c>
       <c r="L170" t="n">
         <v>43.93453482363842</v>
@@ -16976,7 +16976,7 @@
         <v>31.10432393883969</v>
       </c>
       <c r="O170" t="n">
-        <v>120</v>
+        <v>77.98458998395874</v>
       </c>
       <c r="P170" t="n">
         <v>5.628787421921748</v>
@@ -17044,7 +17044,7 @@
         <v>53.83370737210617</v>
       </c>
       <c r="K171" t="n">
-        <v>88.32842195472395</v>
+        <v>11.67157804527604</v>
       </c>
       <c r="L171" t="n">
         <v>44.47122376294349</v>
@@ -17056,7 +17056,7 @@
         <v>29.71443316866408</v>
       </c>
       <c r="O171" t="n">
-        <v>120</v>
+        <v>80.2519873776899</v>
       </c>
       <c r="P171" t="n">
         <v>5.832559329431546</v>
@@ -17124,7 +17124,7 @@
         <v>54.63463657418399</v>
       </c>
       <c r="K172" t="n">
-        <v>93.38937265718774</v>
+        <v>6.61062734281227</v>
       </c>
       <c r="L172" t="n">
         <v>45.0474761310949</v>
@@ -17136,7 +17136,7 @@
         <v>31.34966282435456</v>
       </c>
       <c r="O172" t="n">
-        <v>120</v>
+        <v>81.59459561876628</v>
       </c>
       <c r="P172" t="n">
         <v>8.605288141215626</v>
@@ -17204,7 +17204,7 @@
         <v>55.8999335802235</v>
       </c>
       <c r="K173" t="n">
-        <v>87.14326254800187</v>
+        <v>12.85673745199814</v>
       </c>
       <c r="L173" t="n">
         <v>45.58416507039998</v>
@@ -17216,7 +17216,7 @@
         <v>31.71427252858725</v>
       </c>
       <c r="O173" t="n">
-        <v>120</v>
+        <v>85.44267016362484</v>
       </c>
       <c r="P173" t="n">
         <v>7.909387162739168</v>
@@ -17284,7 +17284,7 @@
         <v>57.30255219410274</v>
       </c>
       <c r="K174" t="n">
-        <v>77.25736106159651</v>
+        <v>22.74263893840348</v>
       </c>
       <c r="L174" t="n">
         <v>45.99351348747959</v>
@@ -17296,7 +17296,7 @@
         <v>32.06373667439</v>
       </c>
       <c r="O174" t="n">
-        <v>94.7229044231309</v>
+        <v>86.10987226220439</v>
       </c>
       <c r="P174" t="n">
         <v>7.365231588894659</v>
@@ -20610,7 +20610,7 @@
         </is>
       </c>
       <c r="B164" t="n">
-        <v>77.25736106159651</v>
+        <v>22.74263893840348</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -20630,7 +20630,7 @@
         </is>
       </c>
       <c r="B165" t="n">
-        <v>68.94527080678576</v>
+        <v>31.05472919321425</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
@@ -20650,7 +20650,7 @@
         </is>
       </c>
       <c r="B166" t="n">
-        <v>74.71757089484051</v>
+        <v>25.28242910515949</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -20670,7 +20670,7 @@
         </is>
       </c>
       <c r="B167" t="n">
-        <v>68.95402353110227</v>
+        <v>31.04597646889773</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
@@ -20690,7 +20690,7 @@
         </is>
       </c>
       <c r="B168" t="n">
-        <v>77.61772592998518</v>
+        <v>22.38227407001482</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -20710,7 +20710,7 @@
         </is>
       </c>
       <c r="B169" t="n">
-        <v>84.31811353379777</v>
+        <v>15.68188646620223</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -20730,7 +20730,7 @@
         </is>
       </c>
       <c r="B170" t="n">
-        <v>64.95460177868776</v>
+        <v>35.04539822131224</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
@@ -20750,7 +20750,7 @@
         </is>
       </c>
       <c r="B171" t="n">
-        <v>84.76120265002956</v>
+        <v>15.23879734997043</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
@@ -20770,7 +20770,7 @@
         </is>
       </c>
       <c r="B172" t="n">
-        <v>86.3823010876974</v>
+        <v>13.6176989123026</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -20790,7 +20790,7 @@
         </is>
       </c>
       <c r="B173" t="n">
-        <v>86.67320809793419</v>
+        <v>13.3267919020658</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -20810,7 +20810,7 @@
         </is>
       </c>
       <c r="B174" t="n">
-        <v>75.3277305538721</v>
+        <v>24.67226944612789</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
@@ -20830,7 +20830,7 @@
         </is>
       </c>
       <c r="B175" t="n">
-        <v>74.29556804706576</v>
+        <v>25.70443195293425</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
@@ -20850,7 +20850,7 @@
         </is>
       </c>
       <c r="B176" t="n">
-        <v>78.90147268563315</v>
+        <v>21.09852731436684</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
@@ -20870,7 +20870,7 @@
         </is>
       </c>
       <c r="B177" t="n">
-        <v>81.85372220732324</v>
+        <v>18.14627779267676</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -20890,7 +20890,7 @@
         </is>
       </c>
       <c r="B178" t="n">
-        <v>74.55092629673469</v>
+        <v>25.44907370326531</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
@@ -20910,7 +20910,7 @@
         </is>
       </c>
       <c r="B179" t="n">
-        <v>60.90453685453214</v>
+        <v>39.09546314546786</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
@@ -20930,7 +20930,7 @@
         </is>
       </c>
       <c r="B180" t="n">
-        <v>76.42120355871066</v>
+        <v>23.57879644128934</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
@@ -20950,7 +20950,7 @@
         </is>
       </c>
       <c r="B181" t="n">
-        <v>76.40913520009576</v>
+        <v>23.59086479990423</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -22050,7 +22050,7 @@
         </is>
       </c>
       <c r="B236" t="n">
-        <v>94.7229044231309</v>
+        <v>86.10987226220439</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -22070,7 +22070,7 @@
         </is>
       </c>
       <c r="B237" t="n">
-        <v>77.0878139473048</v>
+        <v>77.3968668590511</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
@@ -22090,7 +22090,7 @@
         </is>
       </c>
       <c r="B238" t="n">
-        <v>75.80928946754145</v>
+        <v>70.94532874221099</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
@@ -22110,7 +22110,7 @@
         </is>
       </c>
       <c r="B239" t="n">
-        <v>74.74459713480438</v>
+        <v>68.89903839818906</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -22130,7 +22130,7 @@
         </is>
       </c>
       <c r="B240" t="n">
-        <v>60.30862072738036</v>
+        <v>56.94721373950999</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
@@ -22150,7 +22150,7 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>98.39398574590119</v>
+        <v>94.22924626856788</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
@@ -22170,7 +22170,7 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>82.88287348593843</v>
+        <v>78.56973512025898</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
@@ -22190,7 +22190,7 @@
         </is>
       </c>
       <c r="B243" t="n">
-        <v>86.29437703592798</v>
+        <v>82.72358719006965</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
@@ -22210,7 +22210,7 @@
         </is>
       </c>
       <c r="B244" t="n">
-        <v>72.21073230111311</v>
+        <v>62.34228258567671</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
@@ -22230,7 +22230,7 @@
         </is>
       </c>
       <c r="B245" t="n">
-        <v>84.00232685784536</v>
+        <v>78.42455029808916</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
@@ -22250,7 +22250,7 @@
         </is>
       </c>
       <c r="B246" t="n">
-        <v>74.05267842989197</v>
+        <v>70.14494870020187</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
@@ -22270,7 +22270,7 @@
         </is>
       </c>
       <c r="B247" t="n">
-        <v>61.84291256642111</v>
+        <v>58.84586754215799</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -22290,7 +22290,7 @@
         </is>
       </c>
       <c r="B248" t="n">
-        <v>84.81599693137701</v>
+        <v>83.57794325020366</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
@@ -22310,7 +22310,7 @@
         </is>
       </c>
       <c r="B249" t="n">
-        <v>81.94188148849634</v>
+        <v>77.21182469990407</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
@@ -22330,7 +22330,7 @@
         </is>
       </c>
       <c r="B250" t="n">
-        <v>74.54824565803419</v>
+        <v>70.62244278399331</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -22350,7 +22350,7 @@
         </is>
       </c>
       <c r="B251" t="n">
-        <v>83.94024166482441</v>
+        <v>77.49636351428153</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
@@ -22370,7 +22370,7 @@
         </is>
       </c>
       <c r="B252" t="n">
-        <v>83.21288941861825</v>
+        <v>78.33691231031122</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -22390,7 +22390,7 @@
         </is>
       </c>
       <c r="B253" t="n">
-        <v>93.79286950661518</v>
+        <v>88.41022219930377</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>

</xml_diff>